<commit_message>
Ajustes de versão e processo de agrupamento no email
</commit_message>
<xml_diff>
--- a/inputs/base_emails/Base_emails.xlsx
+++ b/inputs/base_emails/Base_emails.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://flytour-my.sharepoint.com/personal/nicolas_cavalcante_flytour_com_br/Documents/Documentos/GitHub/projeto-conciliacao_ebta/inputs/base_emails/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="202" documentId="13_ncr:1_{DDD36486-E38A-45A0-A02C-30309960971C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BF202B92-9FBD-4D88-AF10-0EB3873EA2C6}"/>
+  <xr:revisionPtr revIDLastSave="208" documentId="13_ncr:1_{DDD36486-E38A-45A0-A02C-30309960971C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{33CA1C30-98B0-4BED-9DC3-01110EAF3C22}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CE0543A2-C287-48AB-86E0-EEF591E298AA}"/>
   </bookViews>
@@ -5629,7 +5629,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1273B727-18F5-477A-913A-0C391C249E0F}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:AA419"/>
   <sheetFormatPr defaultColWidth="39.33203125" defaultRowHeight="16.2" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
@@ -5741,7 +5740,7 @@
         <v>1645</v>
       </c>
     </row>
-    <row r="2" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
         <v>22</v>
       </c>
@@ -5818,7 +5817,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="3" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
         <v>43</v>
       </c>
@@ -5901,7 +5900,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="4" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>57</v>
       </c>
@@ -5978,7 +5977,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="5" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>66</v>
       </c>
@@ -6055,7 +6054,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="6" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>70</v>
       </c>
@@ -6132,7 +6131,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="7" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
         <v>76</v>
       </c>
@@ -6209,7 +6208,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="8" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
         <v>79</v>
       </c>
@@ -6286,7 +6285,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="9" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
         <v>92</v>
       </c>
@@ -6363,7 +6362,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="10" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
         <v>94</v>
       </c>
@@ -6440,7 +6439,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="11" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
         <v>100</v>
       </c>
@@ -6517,7 +6516,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="12" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="s">
         <v>102</v>
       </c>
@@ -6594,7 +6593,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="13" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="9" t="s">
         <v>108</v>
       </c>
@@ -6671,7 +6670,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="14" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="9" t="s">
         <v>111</v>
       </c>
@@ -6748,7 +6747,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="15" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="9" t="s">
         <v>111</v>
       </c>
@@ -6825,7 +6824,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="16" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="9" t="s">
         <v>119</v>
       </c>
@@ -6902,7 +6901,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="17" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="9" t="s">
         <v>119</v>
       </c>
@@ -6979,7 +6978,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="18" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
         <v>127</v>
       </c>
@@ -7056,7 +7055,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="19" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
         <v>127</v>
       </c>
@@ -7133,7 +7132,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="20" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="6" t="s">
         <v>136</v>
       </c>
@@ -7207,7 +7206,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="21" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6" t="s">
         <v>150</v>
       </c>
@@ -7281,7 +7280,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="22" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="6" t="s">
         <v>153</v>
       </c>
@@ -7355,7 +7354,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="23" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="6" t="s">
         <v>156</v>
       </c>
@@ -7429,7 +7428,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="24" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="6" t="s">
         <v>167</v>
       </c>
@@ -7503,7 +7502,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="25" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="6" t="s">
         <v>170</v>
       </c>
@@ -7577,7 +7576,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="26" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="6" t="s">
         <v>173</v>
       </c>
@@ -7651,7 +7650,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="27" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
         <v>183</v>
       </c>
@@ -7725,7 +7724,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="28" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
         <v>186</v>
       </c>
@@ -7799,7 +7798,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="29" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
         <v>188</v>
       </c>
@@ -7873,7 +7872,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="30" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
         <v>191</v>
       </c>
@@ -7947,7 +7946,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="31" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="5" t="s">
         <v>194</v>
       </c>
@@ -8021,7 +8020,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="32" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="8" t="s">
         <v>196</v>
       </c>
@@ -8095,7 +8094,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="33" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
         <v>202</v>
       </c>
@@ -8169,7 +8168,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="34" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="8" t="s">
         <v>205</v>
       </c>
@@ -8243,7 +8242,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="35" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="5" t="s">
         <v>214</v>
       </c>
@@ -8317,7 +8316,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="36" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="5" t="s">
         <v>217</v>
       </c>
@@ -8391,7 +8390,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="37" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="6" t="s">
         <v>229</v>
       </c>
@@ -8465,7 +8464,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="38" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="5" t="s">
         <v>233</v>
       </c>
@@ -8539,7 +8538,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="39" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="5" t="s">
         <v>237</v>
       </c>
@@ -8607,7 +8606,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="40" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="5" t="s">
         <v>251</v>
       </c>
@@ -8675,7 +8674,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="41" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="5" t="s">
         <v>253</v>
       </c>
@@ -8746,7 +8745,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="42" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="5" t="s">
         <v>260</v>
       </c>
@@ -8814,7 +8813,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="43" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="5" t="s">
         <v>268</v>
       </c>
@@ -8882,7 +8881,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="44" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="5" t="s">
         <v>272</v>
       </c>
@@ -8950,7 +8949,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="45" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="5" t="s">
         <v>275</v>
       </c>
@@ -9018,7 +9017,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="46" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="5" t="s">
         <v>276</v>
       </c>
@@ -9086,7 +9085,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="47" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="5" t="s">
         <v>280</v>
       </c>
@@ -9160,7 +9159,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="48" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="5" t="s">
         <v>280</v>
       </c>
@@ -9234,7 +9233,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="49" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="5" t="s">
         <v>292</v>
       </c>
@@ -9308,7 +9307,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="50" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="5" t="s">
         <v>297</v>
       </c>
@@ -9385,7 +9384,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="51" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="9" t="s">
         <v>305</v>
       </c>
@@ -9457,7 +9456,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="52" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="9" t="s">
         <v>310</v>
       </c>
@@ -9531,7 +9530,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="53" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="9" t="s">
         <v>310</v>
       </c>
@@ -9605,7 +9604,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="54" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="9" t="s">
         <v>316</v>
       </c>
@@ -9677,7 +9676,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="55" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="9" t="s">
         <v>321</v>
       </c>
@@ -9749,7 +9748,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="56" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="9" t="s">
         <v>324</v>
       </c>
@@ -9821,7 +9820,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="57" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="9" t="s">
         <v>327</v>
       </c>
@@ -9893,7 +9892,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="58" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="9" t="s">
         <v>329</v>
       </c>
@@ -9965,7 +9964,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="59" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="9" t="s">
         <v>334</v>
       </c>
@@ -10037,7 +10036,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="60" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="9" t="s">
         <v>338</v>
       </c>
@@ -10109,7 +10108,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="61" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="9" t="s">
         <v>340</v>
       </c>
@@ -10181,7 +10180,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="62" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="9" t="s">
         <v>341</v>
       </c>
@@ -10253,7 +10252,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="63" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="9" t="s">
         <v>343</v>
       </c>
@@ -10325,7 +10324,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="64" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="9" t="s">
         <v>347</v>
       </c>
@@ -10397,7 +10396,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="65" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="5" t="s">
         <v>349</v>
       </c>
@@ -10469,7 +10468,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="66" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="5" t="s">
         <v>352</v>
       </c>
@@ -10543,7 +10542,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="67" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="5" t="s">
         <v>360</v>
       </c>
@@ -10617,7 +10616,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="68" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="5" t="s">
         <v>363</v>
       </c>
@@ -10685,7 +10684,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="69" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="5" t="s">
         <v>369</v>
       </c>
@@ -10756,7 +10755,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="70" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="5" t="s">
         <v>376</v>
       </c>
@@ -10824,7 +10823,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="71" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="5" t="s">
         <v>382</v>
       </c>
@@ -10892,7 +10891,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="72" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="5" t="s">
         <v>386</v>
       </c>
@@ -10966,7 +10965,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="73" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="5" t="s">
         <v>386</v>
       </c>
@@ -11040,7 +11039,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="74" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="5" t="s">
         <v>386</v>
       </c>
@@ -11114,7 +11113,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="75" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="5" t="s">
         <v>386</v>
       </c>
@@ -11186,7 +11185,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="76" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="5" t="s">
         <v>386</v>
       </c>
@@ -11258,7 +11257,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="77" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" s="5" t="s">
         <v>404</v>
       </c>
@@ -11326,7 +11325,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="78" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" s="5" t="s">
         <v>410</v>
       </c>
@@ -11394,7 +11393,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="79" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="5" t="s">
         <v>412</v>
       </c>
@@ -11466,7 +11465,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="80" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" s="5" t="s">
         <v>412</v>
       </c>
@@ -11538,7 +11537,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="81" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A81" s="9" t="s">
         <v>421</v>
       </c>
@@ -11612,7 +11611,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="82" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="9" t="s">
         <v>421</v>
       </c>
@@ -11686,7 +11685,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="83" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A83" s="9" t="s">
         <v>429</v>
       </c>
@@ -11760,7 +11759,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="84" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A84" s="9" t="s">
         <v>429</v>
       </c>
@@ -11834,7 +11833,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="85" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A85" s="9" t="s">
         <v>435</v>
       </c>
@@ -11906,7 +11905,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="86" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A86" s="9" t="s">
         <v>441</v>
       </c>
@@ -11978,7 +11977,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="87" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A87" s="9" t="s">
         <v>447</v>
       </c>
@@ -12050,7 +12049,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="88" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A88" s="9" t="s">
         <v>449</v>
       </c>
@@ -12124,7 +12123,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="89" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A89" s="9" t="s">
         <v>456</v>
       </c>
@@ -12194,7 +12193,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="90" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" s="9" t="s">
         <v>461</v>
       </c>
@@ -12266,7 +12265,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="91" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A91" s="9" t="s">
         <v>469</v>
       </c>
@@ -12340,7 +12339,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="92" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A92" s="9" t="s">
         <v>475</v>
       </c>
@@ -12414,7 +12413,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="93" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A93" s="9" t="s">
         <v>477</v>
       </c>
@@ -12488,7 +12487,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="94" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" s="9" t="s">
         <v>482</v>
       </c>
@@ -12560,7 +12559,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="95" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A95" s="9" t="s">
         <v>484</v>
       </c>
@@ -12634,7 +12633,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="96" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A96" s="9" t="s">
         <v>484</v>
       </c>
@@ -12708,7 +12707,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="97" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A97" s="9" t="s">
         <v>488</v>
       </c>
@@ -12782,7 +12781,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="98" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" s="9" t="s">
         <v>488</v>
       </c>
@@ -12856,7 +12855,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="99" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A99" s="9" t="s">
         <v>492</v>
       </c>
@@ -12926,7 +12925,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="100" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A100" s="9" t="s">
         <v>492</v>
       </c>
@@ -12996,7 +12995,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="101" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A101" s="5" t="s">
         <v>499</v>
       </c>
@@ -13068,7 +13067,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="102" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A102" s="5" t="s">
         <v>505</v>
       </c>
@@ -13136,7 +13135,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="103" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A103" s="9" t="s">
         <v>512</v>
       </c>
@@ -13210,7 +13209,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="104" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A104" s="9" t="s">
         <v>518</v>
       </c>
@@ -13284,7 +13283,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="105" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A105" s="9" t="s">
         <v>520</v>
       </c>
@@ -13358,7 +13357,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="106" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A106" s="9" t="s">
         <v>524</v>
       </c>
@@ -13432,7 +13431,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="107" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A107" s="9" t="s">
         <v>525</v>
       </c>
@@ -13506,7 +13505,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="108" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A108" s="9" t="s">
         <v>526</v>
       </c>
@@ -13580,7 +13579,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="109" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A109" s="9" t="s">
         <v>527</v>
       </c>
@@ -13654,7 +13653,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="110" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A110" s="9" t="s">
         <v>533</v>
       </c>
@@ -13728,7 +13727,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="111" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A111" s="9" t="s">
         <v>536</v>
       </c>
@@ -13802,7 +13801,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="112" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A112" s="9" t="s">
         <v>543</v>
       </c>
@@ -13876,7 +13875,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="113" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A113" s="9" t="s">
         <v>546</v>
       </c>
@@ -13950,7 +13949,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="114" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A114" s="9" t="s">
         <v>551</v>
       </c>
@@ -14024,7 +14023,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="115" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A115" s="9" t="s">
         <v>554</v>
       </c>
@@ -14098,7 +14097,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="116" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A116" s="9" t="s">
         <v>555</v>
       </c>
@@ -14172,7 +14171,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="117" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A117" s="9" t="s">
         <v>557</v>
       </c>
@@ -14246,7 +14245,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="118" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A118" s="9" t="s">
         <v>558</v>
       </c>
@@ -14320,7 +14319,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="119" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A119" s="9" t="s">
         <v>559</v>
       </c>
@@ -14394,7 +14393,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="120" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A120" s="9" t="s">
         <v>562</v>
       </c>
@@ -14468,7 +14467,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="121" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A121" s="9" t="s">
         <v>563</v>
       </c>
@@ -14542,7 +14541,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="122" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A122" s="9" t="s">
         <v>564</v>
       </c>
@@ -14616,7 +14615,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="123" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A123" s="9" t="s">
         <v>565</v>
       </c>
@@ -14690,7 +14689,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="124" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A124" s="9" t="s">
         <v>567</v>
       </c>
@@ -14764,7 +14763,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="125" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A125" s="9" t="s">
         <v>568</v>
       </c>
@@ -14838,7 +14837,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="126" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A126" s="9" t="s">
         <v>569</v>
       </c>
@@ -14912,7 +14911,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="127" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A127" s="9" t="s">
         <v>570</v>
       </c>
@@ -14986,7 +14985,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="128" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A128" s="9" t="s">
         <v>571</v>
       </c>
@@ -15060,7 +15059,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="129" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A129" s="9" t="s">
         <v>572</v>
       </c>
@@ -15134,7 +15133,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="130" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A130" s="9" t="s">
         <v>573</v>
       </c>
@@ -15208,7 +15207,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="131" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A131" s="9" t="s">
         <v>574</v>
       </c>
@@ -15282,7 +15281,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="132" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A132" s="9" t="s">
         <v>575</v>
       </c>
@@ -15356,7 +15355,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="133" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A133" s="9" t="s">
         <v>576</v>
       </c>
@@ -15428,7 +15427,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="134" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A134" s="11" t="s">
         <v>582</v>
       </c>
@@ -15498,7 +15497,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="135" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A135" s="10" t="s">
         <v>588</v>
       </c>
@@ -15566,7 +15565,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="136" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A136" s="10" t="s">
         <v>592</v>
       </c>
@@ -15634,7 +15633,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="137" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A137" s="10" t="s">
         <v>593</v>
       </c>
@@ -15702,7 +15701,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="138" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A138" s="10" t="s">
         <v>605</v>
       </c>
@@ -15770,7 +15769,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="139" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A139" s="10" t="s">
         <v>612</v>
       </c>
@@ -15832,7 +15831,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="140" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A140" s="10" t="s">
         <v>615</v>
       </c>
@@ -15894,7 +15893,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="141" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A141" s="10" t="s">
         <v>616</v>
       </c>
@@ -15956,7 +15955,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="142" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A142" s="10" t="s">
         <v>617</v>
       </c>
@@ -16018,7 +16017,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="143" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A143" s="10" t="s">
         <v>618</v>
       </c>
@@ -16080,7 +16079,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="144" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A144" s="10" t="s">
         <v>619</v>
       </c>
@@ -16142,7 +16141,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="145" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A145" s="10" t="s">
         <v>620</v>
       </c>
@@ -16204,7 +16203,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="146" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A146" s="10" t="s">
         <v>621</v>
       </c>
@@ -16266,7 +16265,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="147" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A147" s="10" t="s">
         <v>622</v>
       </c>
@@ -16328,7 +16327,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="148" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A148" s="10" t="s">
         <v>623</v>
       </c>
@@ -16390,7 +16389,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="149" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A149" s="10" t="s">
         <v>624</v>
       </c>
@@ -16452,7 +16451,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="150" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A150" s="10" t="s">
         <v>625</v>
       </c>
@@ -16514,7 +16513,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="151" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A151" s="10" t="s">
         <v>626</v>
       </c>
@@ -16576,7 +16575,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="152" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A152" s="10" t="s">
         <v>627</v>
       </c>
@@ -16638,7 +16637,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="153" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A153" s="10" t="s">
         <v>628</v>
       </c>
@@ -16700,7 +16699,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="154" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A154" s="10" t="s">
         <v>629</v>
       </c>
@@ -16762,7 +16761,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="155" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A155" s="10" t="s">
         <v>630</v>
       </c>
@@ -16824,7 +16823,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="156" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A156" s="10" t="s">
         <v>631</v>
       </c>
@@ -16886,7 +16885,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="157" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A157" s="10" t="s">
         <v>632</v>
       </c>
@@ -16948,7 +16947,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="158" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A158" s="10" t="s">
         <v>633</v>
       </c>
@@ -17016,7 +17015,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="159" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A159" s="10" t="s">
         <v>637</v>
       </c>
@@ -17078,7 +17077,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="160" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A160" s="10" t="s">
         <v>638</v>
       </c>
@@ -17140,7 +17139,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="161" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A161" s="10" t="s">
         <v>639</v>
       </c>
@@ -17202,7 +17201,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="162" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A162" s="10" t="s">
         <v>640</v>
       </c>
@@ -17264,7 +17263,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="163" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A163" s="10" t="s">
         <v>641</v>
       </c>
@@ -17326,7 +17325,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="164" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A164" s="10" t="s">
         <v>642</v>
       </c>
@@ -17388,7 +17387,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="165" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A165" s="10" t="s">
         <v>643</v>
       </c>
@@ -17450,7 +17449,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="166" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A166" s="10" t="s">
         <v>644</v>
       </c>
@@ -17512,7 +17511,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="167" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A167" s="10" t="s">
         <v>645</v>
       </c>
@@ -17580,7 +17579,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="168" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A168" s="10" t="s">
         <v>651</v>
       </c>
@@ -17648,7 +17647,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="169" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A169" s="10" t="s">
         <v>655</v>
       </c>
@@ -17716,7 +17715,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="170" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A170" s="10" t="s">
         <v>659</v>
       </c>
@@ -17784,7 +17783,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="171" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A171" s="10" t="s">
         <v>661</v>
       </c>
@@ -17852,7 +17851,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="172" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A172" s="10" t="s">
         <v>668</v>
       </c>
@@ -17920,7 +17919,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="173" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A173" s="10" t="s">
         <v>672</v>
       </c>
@@ -17988,7 +17987,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="174" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A174" s="10" t="s">
         <v>678</v>
       </c>
@@ -18056,7 +18055,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="175" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A175" s="15" t="s">
         <v>680</v>
       </c>
@@ -18127,7 +18126,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="176" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A176" s="10" t="s">
         <v>685</v>
       </c>
@@ -18195,7 +18194,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="177" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A177" s="10" t="s">
         <v>693</v>
       </c>
@@ -18334,7 +18333,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="179" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A179" s="10" t="s">
         <v>709</v>
       </c>
@@ -18402,7 +18401,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="180" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A180" s="10" t="s">
         <v>712</v>
       </c>
@@ -18475,7 +18474,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="181" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A181" s="10" t="s">
         <v>717</v>
       </c>
@@ -18545,7 +18544,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="182" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A182" s="10" t="s">
         <v>723</v>
       </c>
@@ -18615,7 +18614,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="183" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A183" s="10" t="s">
         <v>729</v>
       </c>
@@ -18685,7 +18684,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="184" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A184" s="10" t="s">
         <v>741</v>
       </c>
@@ -18755,7 +18754,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="185" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A185" s="10" t="s">
         <v>749</v>
       </c>
@@ -18825,7 +18824,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="186" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A186" s="10" t="s">
         <v>755</v>
       </c>
@@ -18895,7 +18894,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="187" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A187" s="10" t="s">
         <v>761</v>
       </c>
@@ -18965,7 +18964,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="188" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A188" s="10" t="s">
         <v>764</v>
       </c>
@@ -19035,7 +19034,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="189" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A189" s="10" t="s">
         <v>764</v>
       </c>
@@ -19105,7 +19104,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="190" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A190" s="10" t="s">
         <v>770</v>
       </c>
@@ -19175,7 +19174,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="191" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A191" s="10" t="s">
         <v>774</v>
       </c>
@@ -19245,7 +19244,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="192" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A192" s="10" t="s">
         <v>778</v>
       </c>
@@ -19315,7 +19314,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="193" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A193" s="10" t="s">
         <v>782</v>
       </c>
@@ -19385,7 +19384,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="194" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A194" s="10" t="s">
         <v>791</v>
       </c>
@@ -19458,7 +19457,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="195" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A195" s="10" t="s">
         <v>793</v>
       </c>
@@ -19529,7 +19528,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="196" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A196" s="10" t="s">
         <v>793</v>
       </c>
@@ -19600,7 +19599,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="197" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A197" s="10" t="s">
         <v>800</v>
       </c>
@@ -19670,7 +19669,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="198" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A198" s="10" t="s">
         <v>807</v>
       </c>
@@ -19740,7 +19739,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="199" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A199" s="10" t="s">
         <v>807</v>
       </c>
@@ -19810,7 +19809,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="200" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A200" s="10" t="s">
         <v>810</v>
       </c>
@@ -19876,7 +19875,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="201" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A201" s="10" t="s">
         <v>801</v>
       </c>
@@ -19946,7 +19945,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="202" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A202" s="10" t="s">
         <v>813</v>
       </c>
@@ -20089,7 +20088,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="204" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A204" s="10" t="s">
         <v>823</v>
       </c>
@@ -20159,7 +20158,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="205" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A205" s="10" t="s">
         <v>829</v>
       </c>
@@ -20229,7 +20228,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="206" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A206" s="10" t="s">
         <v>833</v>
       </c>
@@ -20302,7 +20301,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="207" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A207" s="10" t="s">
         <v>836</v>
       </c>
@@ -20372,7 +20371,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="208" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A208" s="10" t="s">
         <v>841</v>
       </c>
@@ -20442,7 +20441,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="209" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A209" s="10" t="s">
         <v>847</v>
       </c>
@@ -20512,7 +20511,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="210" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A210" s="10" t="s">
         <v>850</v>
       </c>
@@ -20582,7 +20581,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="211" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A211" s="10" t="s">
         <v>854</v>
       </c>
@@ -20652,7 +20651,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="212" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A212" s="10" t="s">
         <v>857</v>
       </c>
@@ -20725,7 +20724,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="213" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A213" s="10" t="s">
         <v>865</v>
       </c>
@@ -20795,7 +20794,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="214" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A214" s="10" t="s">
         <v>867</v>
       </c>
@@ -20865,7 +20864,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="215" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A215" s="10" t="s">
         <v>873</v>
       </c>
@@ -20935,7 +20934,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="216" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A216" s="10" t="s">
         <v>214</v>
       </c>
@@ -21005,7 +21004,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="217" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A217" s="10" t="s">
         <v>881</v>
       </c>
@@ -21075,7 +21074,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="218" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A218" s="10" t="s">
         <v>891</v>
       </c>
@@ -21145,7 +21144,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="219" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A219" s="10" t="s">
         <v>896</v>
       </c>
@@ -21215,7 +21214,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="220" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A220" s="10" t="s">
         <v>902</v>
       </c>
@@ -21281,7 +21280,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="221" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A221" s="10" t="s">
         <v>904</v>
       </c>
@@ -21351,7 +21350,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="222" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A222" s="10" t="s">
         <v>910</v>
       </c>
@@ -21421,7 +21420,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="223" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A223" s="10" t="s">
         <v>913</v>
       </c>
@@ -21491,7 +21490,7 @@
         <v>1647</v>
       </c>
     </row>
-    <row r="224" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A224" s="10" t="s">
         <v>919</v>
       </c>
@@ -21570,7 +21569,7 @@
         <v>1641</v>
       </c>
     </row>
-    <row r="225" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A225" s="10" t="s">
         <v>925</v>
       </c>
@@ -21637,7 +21636,7 @@
       </c>
       <c r="W225" s="10"/>
     </row>
-    <row r="226" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A226" s="10" t="s">
         <v>925</v>
       </c>
@@ -21704,7 +21703,7 @@
       </c>
       <c r="W226" s="10"/>
     </row>
-    <row r="227" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A227" s="10" t="s">
         <v>930</v>
       </c>
@@ -21771,7 +21770,7 @@
       </c>
       <c r="W227" s="10"/>
     </row>
-    <row r="228" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A228" s="10" t="s">
         <v>936</v>
       </c>
@@ -21838,7 +21837,7 @@
       </c>
       <c r="W228" s="10"/>
     </row>
-    <row r="229" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A229" s="10" t="s">
         <v>940</v>
       </c>
@@ -21905,7 +21904,7 @@
       </c>
       <c r="W229" s="10"/>
     </row>
-    <row r="230" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A230" s="10" t="s">
         <v>946</v>
       </c>
@@ -21972,7 +21971,7 @@
       </c>
       <c r="W230" s="10"/>
     </row>
-    <row r="231" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A231" s="10" t="s">
         <v>950</v>
       </c>
@@ -22039,7 +22038,7 @@
       </c>
       <c r="W231" s="10"/>
     </row>
-    <row r="232" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A232" s="10" t="s">
         <v>953</v>
       </c>
@@ -22106,7 +22105,7 @@
       </c>
       <c r="W232" s="10"/>
     </row>
-    <row r="233" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A233" s="10" t="s">
         <v>959</v>
       </c>
@@ -22179,7 +22178,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="234" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A234" s="10" t="s">
         <v>964</v>
       </c>
@@ -22252,7 +22251,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="235" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A235" s="10" t="s">
         <v>967</v>
       </c>
@@ -22325,7 +22324,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="236" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A236" s="10" t="s">
         <v>970</v>
       </c>
@@ -22392,7 +22391,7 @@
       </c>
       <c r="W236" s="10"/>
     </row>
-    <row r="237" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A237" s="10" t="s">
         <v>976</v>
       </c>
@@ -22459,7 +22458,7 @@
       </c>
       <c r="W237" s="10"/>
     </row>
-    <row r="238" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A238" s="10" t="s">
         <v>979</v>
       </c>
@@ -22538,7 +22537,7 @@
         <v>1641</v>
       </c>
     </row>
-    <row r="239" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A239" s="10" t="s">
         <v>984</v>
       </c>
@@ -22605,7 +22604,7 @@
       </c>
       <c r="W239" s="10"/>
     </row>
-    <row r="240" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A240" s="10" t="s">
         <v>988</v>
       </c>
@@ -22672,7 +22671,7 @@
       </c>
       <c r="W240" s="10"/>
     </row>
-    <row r="241" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A241" s="10" t="s">
         <v>992</v>
       </c>
@@ -22739,7 +22738,7 @@
       </c>
       <c r="W241" s="10"/>
     </row>
-    <row r="242" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A242" s="10" t="s">
         <v>136</v>
       </c>
@@ -22806,7 +22805,7 @@
       </c>
       <c r="W242" s="10"/>
     </row>
-    <row r="243" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A243" s="10" t="s">
         <v>998</v>
       </c>
@@ -22873,7 +22872,7 @@
       </c>
       <c r="W243" s="10"/>
     </row>
-    <row r="244" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A244" s="10" t="s">
         <v>1001</v>
       </c>
@@ -22940,7 +22939,7 @@
       </c>
       <c r="W244" s="10"/>
     </row>
-    <row r="245" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A245" s="10" t="s">
         <v>1004</v>
       </c>
@@ -23007,7 +23006,7 @@
       </c>
       <c r="W245" s="10"/>
     </row>
-    <row r="246" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A246" s="10" t="s">
         <v>1007</v>
       </c>
@@ -23074,7 +23073,7 @@
       </c>
       <c r="W246" s="10"/>
     </row>
-    <row r="247" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A247" s="10" t="s">
         <v>1013</v>
       </c>
@@ -23141,7 +23140,7 @@
       </c>
       <c r="W247" s="10"/>
     </row>
-    <row r="248" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A248" s="10" t="s">
         <v>1016</v>
       </c>
@@ -23208,7 +23207,7 @@
       </c>
       <c r="W248" s="10"/>
     </row>
-    <row r="249" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A249" s="10" t="s">
         <v>1022</v>
       </c>
@@ -23275,7 +23274,7 @@
       </c>
       <c r="W249" s="10"/>
     </row>
-    <row r="250" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A250" s="10" t="s">
         <v>1026</v>
       </c>
@@ -23342,7 +23341,7 @@
       </c>
       <c r="W250" s="10"/>
     </row>
-    <row r="251" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A251" s="10" t="s">
         <v>1032</v>
       </c>
@@ -23409,7 +23408,7 @@
       </c>
       <c r="W251" s="10"/>
     </row>
-    <row r="252" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A252" s="10" t="s">
         <v>1040</v>
       </c>
@@ -23476,7 +23475,7 @@
       </c>
       <c r="W252" s="10"/>
     </row>
-    <row r="253" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A253" s="10" t="s">
         <v>1044</v>
       </c>
@@ -23839,7 +23838,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="258" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A258" s="10" t="s">
         <v>1067</v>
       </c>
@@ -23906,7 +23905,7 @@
       </c>
       <c r="W258" s="10"/>
     </row>
-    <row r="259" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A259" s="10" t="s">
         <v>1069</v>
       </c>
@@ -23973,7 +23972,7 @@
       </c>
       <c r="W259" s="10"/>
     </row>
-    <row r="260" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A260" s="10" t="s">
         <v>1074</v>
       </c>
@@ -24040,7 +24039,7 @@
       </c>
       <c r="W260" s="10"/>
     </row>
-    <row r="261" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A261" s="10" t="s">
         <v>1080</v>
       </c>
@@ -24107,7 +24106,7 @@
       </c>
       <c r="W261" s="10"/>
     </row>
-    <row r="262" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A262" s="10" t="s">
         <v>1084</v>
       </c>
@@ -24174,7 +24173,7 @@
       </c>
       <c r="W262" s="10"/>
     </row>
-    <row r="263" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A263" s="10" t="s">
         <v>1086</v>
       </c>
@@ -24241,7 +24240,7 @@
       </c>
       <c r="W263" s="10"/>
     </row>
-    <row r="264" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A264" s="10" t="s">
         <v>1093</v>
       </c>
@@ -24308,7 +24307,7 @@
       </c>
       <c r="W264" s="10"/>
     </row>
-    <row r="265" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A265" s="10" t="s">
         <v>1095</v>
       </c>
@@ -24381,7 +24380,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="266" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A266" s="10" t="s">
         <v>1098</v>
       </c>
@@ -24600,7 +24599,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="269" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A269" s="10" t="s">
         <v>1109</v>
       </c>
@@ -24667,7 +24666,7 @@
       </c>
       <c r="W269" s="10"/>
     </row>
-    <row r="270" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A270" s="10" t="s">
         <v>1115</v>
       </c>
@@ -24734,7 +24733,7 @@
       </c>
       <c r="W270" s="10"/>
     </row>
-    <row r="271" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A271" s="10" t="s">
         <v>1121</v>
       </c>
@@ -24801,7 +24800,7 @@
       </c>
       <c r="W271" s="10"/>
     </row>
-    <row r="272" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A272" s="10" t="s">
         <v>1127</v>
       </c>
@@ -24868,7 +24867,7 @@
       </c>
       <c r="W272" s="10"/>
     </row>
-    <row r="273" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A273" s="10" t="s">
         <v>1133</v>
       </c>
@@ -24941,7 +24940,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="274" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A274" s="10" t="s">
         <v>1138</v>
       </c>
@@ -25008,7 +25007,7 @@
       </c>
       <c r="W274" s="10"/>
     </row>
-    <row r="275" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A275" s="10" t="s">
         <v>1142</v>
       </c>
@@ -25075,7 +25074,7 @@
       </c>
       <c r="W275" s="10"/>
     </row>
-    <row r="276" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A276" s="10" t="s">
         <v>1148</v>
       </c>
@@ -25142,7 +25141,7 @@
       </c>
       <c r="W276" s="10"/>
     </row>
-    <row r="277" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A277" s="10" t="s">
         <v>1152</v>
       </c>
@@ -25209,7 +25208,7 @@
       </c>
       <c r="W277" s="10"/>
     </row>
-    <row r="278" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A278" s="10" t="s">
         <v>1158</v>
       </c>
@@ -25276,7 +25275,7 @@
       </c>
       <c r="W278" s="10"/>
     </row>
-    <row r="279" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A279" s="10" t="s">
         <v>1165</v>
       </c>
@@ -25349,7 +25348,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="280" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A280" s="10" t="s">
         <v>1167</v>
       </c>
@@ -25416,7 +25415,7 @@
       </c>
       <c r="W280" s="10"/>
     </row>
-    <row r="281" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A281" s="10" t="s">
         <v>1170</v>
       </c>
@@ -25483,7 +25482,7 @@
       </c>
       <c r="W281" s="10"/>
     </row>
-    <row r="282" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A282" s="10" t="s">
         <v>1174</v>
       </c>
@@ -25550,7 +25549,7 @@
       </c>
       <c r="W282" s="10"/>
     </row>
-    <row r="283" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A283" s="10" t="s">
         <v>1176</v>
       </c>
@@ -25617,7 +25616,7 @@
       </c>
       <c r="W283" s="10"/>
     </row>
-    <row r="284" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A284" s="10" t="s">
         <v>1181</v>
       </c>
@@ -25684,7 +25683,7 @@
       </c>
       <c r="W284" s="10"/>
     </row>
-    <row r="285" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A285" s="10" t="s">
         <v>1184</v>
       </c>
@@ -25751,7 +25750,7 @@
       </c>
       <c r="W285" s="10"/>
     </row>
-    <row r="286" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A286" s="10" t="s">
         <v>1187</v>
       </c>
@@ -25967,7 +25966,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="289" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A289" s="10" t="s">
         <v>1198</v>
       </c>
@@ -26245,7 +26244,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="293" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A293" s="10" t="s">
         <v>1211</v>
       </c>
@@ -26391,7 +26390,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="295" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A295" s="10" t="s">
         <v>1218</v>
       </c>
@@ -26458,7 +26457,7 @@
       </c>
       <c r="W295" s="10"/>
     </row>
-    <row r="296" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A296" s="10" t="s">
         <v>1221</v>
       </c>
@@ -26525,7 +26524,7 @@
       </c>
       <c r="W296" s="10"/>
     </row>
-    <row r="297" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A297" s="10" t="s">
         <v>1224</v>
       </c>
@@ -26592,7 +26591,7 @@
       </c>
       <c r="W297" s="10"/>
     </row>
-    <row r="298" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A298" s="10" t="s">
         <v>1228</v>
       </c>
@@ -26659,7 +26658,7 @@
       </c>
       <c r="W298" s="10"/>
     </row>
-    <row r="299" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A299" s="10" t="s">
         <v>1232</v>
       </c>
@@ -26726,7 +26725,7 @@
       </c>
       <c r="W299" s="10"/>
     </row>
-    <row r="300" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A300" s="10" t="s">
         <v>1233</v>
       </c>
@@ -26793,7 +26792,7 @@
       </c>
       <c r="W300" s="10"/>
     </row>
-    <row r="301" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A301" s="10" t="s">
         <v>1237</v>
       </c>
@@ -26866,7 +26865,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="302" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A302" s="10" t="s">
         <v>1241</v>
       </c>
@@ -26933,7 +26932,7 @@
       </c>
       <c r="W302" s="10"/>
     </row>
-    <row r="303" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A303" s="10" t="s">
         <v>1246</v>
       </c>
@@ -27000,7 +26999,7 @@
       </c>
       <c r="W303" s="10"/>
     </row>
-    <row r="304" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A304" s="10" t="s">
         <v>823</v>
       </c>
@@ -27067,7 +27066,7 @@
       </c>
       <c r="W304" s="10"/>
     </row>
-    <row r="305" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A305" s="10" t="s">
         <v>1252</v>
       </c>
@@ -27130,7 +27129,7 @@
       </c>
       <c r="W305" s="10"/>
     </row>
-    <row r="306" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A306" s="10" t="s">
         <v>1254</v>
       </c>
@@ -27197,7 +27196,7 @@
       </c>
       <c r="W306" s="10"/>
     </row>
-    <row r="307" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A307" s="10" t="s">
         <v>1257</v>
       </c>
@@ -27260,7 +27259,7 @@
       </c>
       <c r="W307" s="10"/>
     </row>
-    <row r="308" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A308" s="10" t="s">
         <v>1259</v>
       </c>
@@ -27323,7 +27322,7 @@
       </c>
       <c r="W308" s="10"/>
     </row>
-    <row r="309" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="309" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A309" s="10" t="s">
         <v>1261</v>
       </c>
@@ -27386,7 +27385,7 @@
       </c>
       <c r="W309" s="10"/>
     </row>
-    <row r="310" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="310" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A310" s="10" t="s">
         <v>1263</v>
       </c>
@@ -27449,7 +27448,7 @@
       </c>
       <c r="W310" s="10"/>
     </row>
-    <row r="311" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="311" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A311" s="10" t="s">
         <v>1265</v>
       </c>
@@ -27516,7 +27515,7 @@
       </c>
       <c r="W311" s="10"/>
     </row>
-    <row r="312" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="312" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A312" s="10" t="s">
         <v>233</v>
       </c>
@@ -27579,7 +27578,7 @@
       </c>
       <c r="W312" s="10"/>
     </row>
-    <row r="313" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="313" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A313" s="10" t="s">
         <v>1273</v>
       </c>
@@ -27646,7 +27645,7 @@
       </c>
       <c r="W313" s="10"/>
     </row>
-    <row r="314" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="314" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A314" s="10" t="s">
         <v>1279</v>
       </c>
@@ -27714,7 +27713,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="315" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="315" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A315" s="10" t="s">
         <v>1288</v>
       </c>
@@ -27782,7 +27781,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="316" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="316" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A316" s="10" t="s">
         <v>1292</v>
       </c>
@@ -27848,7 +27847,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="317" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="317" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A317" s="10" t="s">
         <v>1294</v>
       </c>
@@ -27915,7 +27914,7 @@
       </c>
       <c r="W317" s="10"/>
     </row>
-    <row r="318" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="318" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A318" s="10" t="s">
         <v>1298</v>
       </c>
@@ -27982,7 +27981,7 @@
       </c>
       <c r="W318" s="10"/>
     </row>
-    <row r="319" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="319" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A319" s="10" t="s">
         <v>1298</v>
       </c>
@@ -28118,7 +28117,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="321" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="321" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A321" s="10" t="s">
         <v>1309</v>
       </c>
@@ -28185,7 +28184,7 @@
       </c>
       <c r="W321" s="10"/>
     </row>
-    <row r="322" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="322" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A322" s="10" t="s">
         <v>1315</v>
       </c>
@@ -28248,7 +28247,7 @@
       </c>
       <c r="W322" s="10"/>
     </row>
-    <row r="323" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="323" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A323" s="10" t="s">
         <v>1317</v>
       </c>
@@ -28315,7 +28314,7 @@
       </c>
       <c r="W323" s="10"/>
     </row>
-    <row r="324" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="324" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A324" s="10" t="s">
         <v>1321</v>
       </c>
@@ -28382,7 +28381,7 @@
       </c>
       <c r="W324" s="10"/>
     </row>
-    <row r="325" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="325" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A325" s="10" t="s">
         <v>1325</v>
       </c>
@@ -28451,7 +28450,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="326" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="326" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A326" s="10" t="s">
         <v>1327</v>
       </c>
@@ -28524,7 +28523,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="327" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="327" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A327" s="10" t="s">
         <v>1331</v>
       </c>
@@ -28593,7 +28592,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="328" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="328" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A328" s="10" t="s">
         <v>1333</v>
       </c>
@@ -28660,7 +28659,7 @@
       </c>
       <c r="W328" s="10"/>
     </row>
-    <row r="329" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="329" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A329" s="10" t="s">
         <v>1337</v>
       </c>
@@ -28727,7 +28726,7 @@
       </c>
       <c r="W329" s="10"/>
     </row>
-    <row r="330" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="330" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A330" s="10" t="s">
         <v>1339</v>
       </c>
@@ -28794,7 +28793,7 @@
       </c>
       <c r="W330" s="10"/>
     </row>
-    <row r="331" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="331" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A331" s="10" t="s">
         <v>1343</v>
       </c>
@@ -28861,7 +28860,7 @@
       </c>
       <c r="W331" s="10"/>
     </row>
-    <row r="332" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="332" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A332" s="10" t="s">
         <v>1347</v>
       </c>
@@ -28928,7 +28927,7 @@
       </c>
       <c r="W332" s="10"/>
     </row>
-    <row r="333" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="333" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A333" s="10" t="s">
         <v>1350</v>
       </c>
@@ -28991,7 +28990,7 @@
       </c>
       <c r="W333" s="10"/>
     </row>
-    <row r="334" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="334" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A334" s="10" t="s">
         <v>1352</v>
       </c>
@@ -29058,7 +29057,7 @@
       </c>
       <c r="W334" s="10"/>
     </row>
-    <row r="335" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="335" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A335" s="10" t="s">
         <v>1356</v>
       </c>
@@ -29121,7 +29120,7 @@
       </c>
       <c r="W335" s="10"/>
     </row>
-    <row r="336" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="336" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A336" s="10" t="s">
         <v>1360</v>
       </c>
@@ -29188,7 +29187,7 @@
       </c>
       <c r="W336" s="10"/>
     </row>
-    <row r="337" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="337" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A337" s="10" t="s">
         <v>1366</v>
       </c>
@@ -29255,7 +29254,7 @@
       </c>
       <c r="W337" s="10"/>
     </row>
-    <row r="338" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="338" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A338" s="10" t="s">
         <v>1370</v>
       </c>
@@ -29322,7 +29321,7 @@
       </c>
       <c r="W338" s="10"/>
     </row>
-    <row r="339" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="339" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A339" s="10" t="s">
         <v>1376</v>
       </c>
@@ -29389,7 +29388,7 @@
       </c>
       <c r="W339" s="10"/>
     </row>
-    <row r="340" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="340" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A340" s="10" t="s">
         <v>1382</v>
       </c>
@@ -29456,7 +29455,7 @@
       </c>
       <c r="W340" s="10"/>
     </row>
-    <row r="341" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="341" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A341" s="10" t="s">
         <v>1007</v>
       </c>
@@ -29523,7 +29522,7 @@
       </c>
       <c r="W341" s="10"/>
     </row>
-    <row r="342" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="342" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A342" s="10" t="s">
         <v>1387</v>
       </c>
@@ -29590,7 +29589,7 @@
       </c>
       <c r="W342" s="10"/>
     </row>
-    <row r="343" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="343" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A343" s="10" t="s">
         <v>1390</v>
       </c>
@@ -29657,7 +29656,7 @@
       </c>
       <c r="W343" s="10"/>
     </row>
-    <row r="344" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="344" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A344" s="10" t="s">
         <v>1391</v>
       </c>
@@ -29724,7 +29723,7 @@
       </c>
       <c r="W344" s="10"/>
     </row>
-    <row r="345" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="345" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A345" s="10" t="s">
         <v>1393</v>
       </c>
@@ -29787,7 +29786,7 @@
       </c>
       <c r="W345" s="10"/>
     </row>
-    <row r="346" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="346" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A346" s="10" t="s">
         <v>1395</v>
       </c>
@@ -29850,7 +29849,7 @@
       </c>
       <c r="W346" s="10"/>
     </row>
-    <row r="347" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="347" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A347" s="10" t="s">
         <v>1397</v>
       </c>
@@ -29917,7 +29916,7 @@
       </c>
       <c r="W347" s="10"/>
     </row>
-    <row r="348" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="348" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A348" s="10" t="s">
         <v>1074</v>
       </c>
@@ -29984,7 +29983,7 @@
       </c>
       <c r="W348" s="10"/>
     </row>
-    <row r="349" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="349" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A349" s="10" t="s">
         <v>1402</v>
       </c>
@@ -30059,7 +30058,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="350" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="350" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A350" s="10" t="s">
         <v>1406</v>
       </c>
@@ -30138,7 +30137,7 @@
         <v>1641</v>
       </c>
     </row>
-    <row r="351" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="351" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A351" s="10" t="s">
         <v>1412</v>
       </c>
@@ -30217,7 +30216,7 @@
         <v>1641</v>
       </c>
     </row>
-    <row r="352" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="352" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A352" s="10" t="s">
         <v>1418</v>
       </c>
@@ -30280,7 +30279,7 @@
       </c>
       <c r="W352" s="10"/>
     </row>
-    <row r="353" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="353" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A353" s="10" t="s">
         <v>1419</v>
       </c>
@@ -30343,7 +30342,7 @@
       </c>
       <c r="W353" s="10"/>
     </row>
-    <row r="354" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="354" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A354" s="10" t="s">
         <v>1421</v>
       </c>
@@ -30410,7 +30409,7 @@
       </c>
       <c r="W354" s="10"/>
     </row>
-    <row r="355" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="355" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A355" s="10" t="s">
         <v>1427</v>
       </c>
@@ -30477,7 +30476,7 @@
       </c>
       <c r="W355" s="10"/>
     </row>
-    <row r="356" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="356" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A356" s="10" t="s">
         <v>1435</v>
       </c>
@@ -30546,7 +30545,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="357" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="357" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A357" s="10" t="s">
         <v>1437</v>
       </c>
@@ -30609,7 +30608,7 @@
       </c>
       <c r="W357" s="10"/>
     </row>
-    <row r="358" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="358" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A358" s="10" t="s">
         <v>1439</v>
       </c>
@@ -30676,7 +30675,7 @@
       </c>
       <c r="W358" s="10"/>
     </row>
-    <row r="359" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="359" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A359" s="10" t="s">
         <v>1444</v>
       </c>
@@ -30739,7 +30738,7 @@
       </c>
       <c r="W359" s="10"/>
     </row>
-    <row r="360" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="360" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A360" s="10" t="s">
         <v>1444</v>
       </c>
@@ -30806,7 +30805,7 @@
       </c>
       <c r="W360" s="10"/>
     </row>
-    <row r="361" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="361" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A361" s="10" t="s">
         <v>1448</v>
       </c>
@@ -30873,7 +30872,7 @@
       </c>
       <c r="W361" s="10"/>
     </row>
-    <row r="362" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="362" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A362" s="10" t="s">
         <v>1448</v>
       </c>
@@ -30940,7 +30939,7 @@
       </c>
       <c r="W362" s="10"/>
     </row>
-    <row r="363" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="363" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A363" s="10" t="s">
         <v>1448</v>
       </c>
@@ -31007,7 +31006,7 @@
       </c>
       <c r="W363" s="10"/>
     </row>
-    <row r="364" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="364" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A364" s="10" t="s">
         <v>1448</v>
       </c>
@@ -31074,7 +31073,7 @@
       </c>
       <c r="W364" s="10"/>
     </row>
-    <row r="365" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="365" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A365" s="10" t="s">
         <v>1456</v>
       </c>
@@ -31139,7 +31138,7 @@
       </c>
       <c r="W365" s="10"/>
     </row>
-    <row r="366" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="366" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A366" s="10" t="s">
         <v>1459</v>
       </c>
@@ -31202,7 +31201,7 @@
       </c>
       <c r="W366" s="10"/>
     </row>
-    <row r="367" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="367" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A367" s="10" t="s">
         <v>1461</v>
       </c>
@@ -31269,7 +31268,7 @@
       </c>
       <c r="W367" s="10"/>
     </row>
-    <row r="368" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="368" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A368" s="10" t="s">
         <v>1465</v>
       </c>
@@ -31336,7 +31335,7 @@
       </c>
       <c r="W368" s="10"/>
     </row>
-    <row r="369" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="369" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A369" s="10" t="s">
         <v>1471</v>
       </c>
@@ -31403,7 +31402,7 @@
       </c>
       <c r="W369" s="10"/>
     </row>
-    <row r="370" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="370" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A370" s="10" t="s">
         <v>1474</v>
       </c>
@@ -31470,7 +31469,7 @@
       </c>
       <c r="W370" s="10"/>
     </row>
-    <row r="371" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="371" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A371" s="10" t="s">
         <v>1477</v>
       </c>
@@ -31537,7 +31536,7 @@
       </c>
       <c r="W371" s="10"/>
     </row>
-    <row r="372" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="372" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A372" s="10" t="s">
         <v>1481</v>
       </c>
@@ -31600,7 +31599,7 @@
       </c>
       <c r="W372" s="10"/>
     </row>
-    <row r="373" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="373" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A373" s="10" t="s">
         <v>1483</v>
       </c>
@@ -31667,7 +31666,7 @@
       </c>
       <c r="W373" s="10"/>
     </row>
-    <row r="374" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="374" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A374" s="10" t="s">
         <v>1489</v>
       </c>
@@ -31734,7 +31733,7 @@
       </c>
       <c r="W374" s="10"/>
     </row>
-    <row r="375" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="375" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A375" s="10" t="s">
         <v>1493</v>
       </c>
@@ -31797,7 +31796,7 @@
       </c>
       <c r="W375" s="10"/>
     </row>
-    <row r="376" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="376" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A376" s="10" t="s">
         <v>1495</v>
       </c>
@@ -31864,7 +31863,7 @@
       </c>
       <c r="W376" s="10"/>
     </row>
-    <row r="377" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="377" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A377" s="10" t="s">
         <v>1498</v>
       </c>
@@ -32004,7 +32003,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="379" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="379" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A379" s="10" t="s">
         <v>1505</v>
       </c>
@@ -32071,7 +32070,7 @@
       </c>
       <c r="W379" s="10"/>
     </row>
-    <row r="380" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="380" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A380" s="10" t="s">
         <v>1507</v>
       </c>
@@ -32134,7 +32133,7 @@
       </c>
       <c r="W380" s="10"/>
     </row>
-    <row r="381" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="381" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A381" s="10" t="s">
         <v>1509</v>
       </c>
@@ -32201,7 +32200,7 @@
       </c>
       <c r="W381" s="10"/>
     </row>
-    <row r="382" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="382" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A382" s="10" t="s">
         <v>1513</v>
       </c>
@@ -32268,7 +32267,7 @@
       </c>
       <c r="W382" s="10"/>
     </row>
-    <row r="383" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="383" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A383" s="10" t="s">
         <v>1516</v>
       </c>
@@ -32331,7 +32330,7 @@
       </c>
       <c r="W383" s="10"/>
     </row>
-    <row r="384" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="384" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A384" s="10" t="s">
         <v>764</v>
       </c>
@@ -32394,7 +32393,7 @@
       </c>
       <c r="W384" s="10"/>
     </row>
-    <row r="385" spans="1:23" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="385" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A385" s="10" t="s">
         <v>1518</v>
       </c>
@@ -32461,7 +32460,7 @@
       </c>
       <c r="W385" s="10"/>
     </row>
-    <row r="386" spans="1:23" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="386" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A386" s="10" t="s">
         <v>1523</v>
       </c>
@@ -32524,7 +32523,7 @@
       </c>
       <c r="W386" s="10"/>
     </row>
-    <row r="387" spans="1:23" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="387" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A387" s="10" t="s">
         <v>1525</v>
       </c>
@@ -32587,7 +32586,7 @@
       </c>
       <c r="W387" s="10"/>
     </row>
-    <row r="388" spans="1:23" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="388" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A388" s="10" t="s">
         <v>1527</v>
       </c>
@@ -32650,7 +32649,7 @@
       </c>
       <c r="W388" s="10"/>
     </row>
-    <row r="389" spans="1:23" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="389" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A389" s="10" t="s">
         <v>1529</v>
       </c>
@@ -32713,7 +32712,7 @@
       </c>
       <c r="W389" s="10"/>
     </row>
-    <row r="390" spans="1:23" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="390" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A390" s="10" t="s">
         <v>1531</v>
       </c>
@@ -32778,7 +32777,7 @@
       </c>
       <c r="W390" s="10"/>
     </row>
-    <row r="391" spans="1:23" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="391" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A391" s="10" t="s">
         <v>989</v>
       </c>
@@ -32845,7 +32844,7 @@
       </c>
       <c r="W391" s="10"/>
     </row>
-    <row r="392" spans="1:23" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="392" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A392" s="10" t="s">
         <v>1537</v>
       </c>
@@ -32912,7 +32911,7 @@
       </c>
       <c r="W392" s="10"/>
     </row>
-    <row r="393" spans="1:23" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="393" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A393" s="10" t="s">
         <v>1540</v>
       </c>
@@ -32979,7 +32978,7 @@
       </c>
       <c r="W393" s="10"/>
     </row>
-    <row r="394" spans="1:23" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="394" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A394" s="10" t="s">
         <v>1546</v>
       </c>
@@ -33046,7 +33045,7 @@
       </c>
       <c r="W394" s="10"/>
     </row>
-    <row r="395" spans="1:23" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="395" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A395" s="10" t="s">
         <v>1550</v>
       </c>
@@ -33113,7 +33112,7 @@
       </c>
       <c r="W395" s="10"/>
     </row>
-    <row r="396" spans="1:23" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="396" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A396" s="10" t="s">
         <v>1553</v>
       </c>
@@ -33180,7 +33179,7 @@
       </c>
       <c r="W396" s="10"/>
     </row>
-    <row r="397" spans="1:23" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="397" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A397" s="10" t="s">
         <v>1559</v>
       </c>
@@ -33247,7 +33246,7 @@
       </c>
       <c r="W397" s="10"/>
     </row>
-    <row r="398" spans="1:23" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="398" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A398" s="10" t="s">
         <v>1562</v>
       </c>
@@ -33314,7 +33313,7 @@
       </c>
       <c r="W398" s="10"/>
     </row>
-    <row r="399" spans="1:23" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="399" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A399" s="10" t="s">
         <v>1568</v>
       </c>
@@ -33377,7 +33376,7 @@
       </c>
       <c r="W399" s="10"/>
     </row>
-    <row r="400" spans="1:23" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="400" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A400" s="10" t="s">
         <v>1570</v>
       </c>
@@ -33444,7 +33443,7 @@
       </c>
       <c r="W400" s="10"/>
     </row>
-    <row r="401" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="401" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A401" s="10" t="s">
         <v>1574</v>
       </c>
@@ -33507,7 +33506,7 @@
       </c>
       <c r="W401" s="10"/>
     </row>
-    <row r="402" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="402" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A402" s="10" t="s">
         <v>1576</v>
       </c>
@@ -33570,7 +33569,7 @@
       </c>
       <c r="W402" s="10"/>
     </row>
-    <row r="403" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="403" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A403" s="10" t="s">
         <v>1582</v>
       </c>
@@ -33633,7 +33632,7 @@
       </c>
       <c r="W403" s="10"/>
     </row>
-    <row r="404" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="404" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A404" s="10" t="s">
         <v>1584</v>
       </c>
@@ -33700,7 +33699,7 @@
       </c>
       <c r="W404" s="10"/>
     </row>
-    <row r="405" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="405" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A405" s="10" t="s">
         <v>1591</v>
       </c>
@@ -33763,7 +33762,7 @@
       </c>
       <c r="W405" s="10"/>
     </row>
-    <row r="406" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="406" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A406" s="10" t="s">
         <v>1593</v>
       </c>
@@ -33830,7 +33829,7 @@
       </c>
       <c r="W406" s="10"/>
     </row>
-    <row r="407" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="407" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A407" s="10" t="s">
         <v>1597</v>
       </c>
@@ -33897,7 +33896,7 @@
       </c>
       <c r="W407" s="10"/>
     </row>
-    <row r="408" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="408" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A408" s="10" t="s">
         <v>1602</v>
       </c>
@@ -33976,7 +33975,7 @@
         <v>1641</v>
       </c>
     </row>
-    <row r="409" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="409" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A409" s="10" t="s">
         <v>1605</v>
       </c>
@@ -34185,7 +34184,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="412" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="412" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A412" s="10" t="s">
         <v>1613</v>
       </c>
@@ -34252,7 +34251,7 @@
       </c>
       <c r="W412" s="10"/>
     </row>
-    <row r="413" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="413" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A413" s="10" t="s">
         <v>1617</v>
       </c>
@@ -34319,7 +34318,7 @@
       </c>
       <c r="W413" s="10"/>
     </row>
-    <row r="414" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="414" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A414" s="10" t="s">
         <v>1621</v>
       </c>
@@ -34386,7 +34385,7 @@
       </c>
       <c r="W414" s="10"/>
     </row>
-    <row r="415" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="415" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A415" s="15" t="s">
         <v>1623</v>
       </c>
@@ -34453,7 +34452,7 @@
       </c>
       <c r="W415" s="15"/>
     </row>
-    <row r="416" spans="1:27" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="416" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A416" s="5" t="s">
         <v>1627</v>
       </c>
@@ -34520,7 +34519,7 @@
       </c>
       <c r="W416" s="5"/>
     </row>
-    <row r="417" spans="1:23" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="417" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A417" s="5" t="s">
         <v>1631</v>
       </c>
@@ -34585,7 +34584,7 @@
       </c>
       <c r="W417" s="5"/>
     </row>
-    <row r="418" spans="1:23" ht="16.2" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="418" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A418" s="5" t="s">
         <v>1634</v>
       </c>
@@ -34656,13 +34655,7 @@
       <c r="A419"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AA418" xr:uid="{1273B727-18F5-477A-913A-0C391C249E0F}">
-    <filterColumn colId="12">
-      <filters>
-        <filter val="DISCOVERY"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:AA418" xr:uid="{1273B727-18F5-477A-913A-0C391C249E0F}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:Z133">
     <sortCondition ref="L2:L133"/>
   </sortState>

</xml_diff>

<commit_message>
Ajustes no envio de email e finalização da regra para os disparos
</commit_message>
<xml_diff>
--- a/inputs/base_emails/Base_emails.xlsx
+++ b/inputs/base_emails/Base_emails.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://flytour-my.sharepoint.com/personal/nicolas_cavalcante_flytour_com_br/Documents/Documentos/GitHub/projeto-conciliacao_ebta/inputs/base_emails/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="208" documentId="13_ncr:1_{DDD36486-E38A-45A0-A02C-30309960971C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{33CA1C30-98B0-4BED-9DC3-01110EAF3C22}"/>
+  <xr:revisionPtr revIDLastSave="297" documentId="13_ncr:1_{DDD36486-E38A-45A0-A02C-30309960971C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BD702769-5BAA-4546-BA57-4BE308ABF36A}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CE0543A2-C287-48AB-86E0-EEF591E298AA}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8293" uniqueCount="1648">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8046" uniqueCount="1645">
   <si>
     <t>Cliente Conciliadora</t>
   </si>
@@ -4982,32 +4982,23 @@
     <t>GERENTE_TESTE</t>
   </si>
   <si>
+    <t>EMAIL_CELULA_TESTE</t>
+  </si>
+  <si>
+    <t>Nº Cliente/COMP</t>
+  </si>
+  <si>
+    <t>nicolas.cavalcante@flytour.com.br</t>
+  </si>
+  <si>
     <t>nathalia.santos@flytour.com.br</t>
-  </si>
-  <si>
-    <t>allan.ribeiro@flytour.com.br</t>
-  </si>
-  <si>
-    <t>karina.deniz@flytour.com.br</t>
-  </si>
-  <si>
-    <t>guilherme.alves@flytour.com.br</t>
-  </si>
-  <si>
-    <t>EMAIL_CELULA_TESTE</t>
-  </si>
-  <si>
-    <t>Nº Cliente/COMP</t>
-  </si>
-  <si>
-    <t>nicolas.cavalcante@flytour.com.br</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -5066,6 +5057,15 @@
     </font>
     <font>
       <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -5163,7 +5163,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -5217,6 +5217,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="4" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -5674,7 +5677,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>1646</v>
+        <v>1642</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>5</v>
@@ -5730,14 +5733,14 @@
       <c r="X1" s="2" t="s">
         <v>1638</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="Y1" s="19" t="s">
         <v>1639</v>
       </c>
       <c r="Z1" s="2" t="s">
         <v>1640</v>
       </c>
       <c r="AA1" s="2" t="s">
-        <v>1645</v>
+        <v>1641</v>
       </c>
     </row>
     <row r="2" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -5810,12 +5813,6 @@
       <c r="W2" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="Z2" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA2" s="18" t="s">
-        <v>1642</v>
-      </c>
     </row>
     <row r="3" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -5887,17 +5884,10 @@
       <c r="W3" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="X3" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="Y3" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="Z3" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA3" s="1" t="s">
-        <v>1647</v>
+      <c r="X3" s="18"/>
+      <c r="Y3" s="18"/>
+      <c r="Z3" t="s">
+        <v>1643</v>
       </c>
     </row>
     <row r="4" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -5970,12 +5960,6 @@
       <c r="W4" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="Z4" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA4" s="18" t="s">
-        <v>1642</v>
-      </c>
     </row>
     <row r="5" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
@@ -6047,12 +6031,6 @@
       <c r="W5" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="Z5" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA5" s="18" t="s">
-        <v>1642</v>
-      </c>
     </row>
     <row r="6" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
@@ -6124,12 +6102,6 @@
       <c r="W6" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="Z6" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA6" s="18" t="s">
-        <v>1642</v>
-      </c>
     </row>
     <row r="7" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
@@ -6201,12 +6173,6 @@
       <c r="W7" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="Z7" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA7" s="18" t="s">
-        <v>1642</v>
-      </c>
     </row>
     <row r="8" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
@@ -6278,12 +6244,6 @@
       <c r="W8" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="Z8" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA8" s="18" t="s">
-        <v>1642</v>
-      </c>
     </row>
     <row r="9" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
@@ -6355,12 +6315,6 @@
       <c r="W9" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="Z9" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA9" s="18" t="s">
-        <v>1642</v>
-      </c>
     </row>
     <row r="10" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
@@ -6432,12 +6386,6 @@
       <c r="W10" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="Z10" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA10" s="18" t="s">
-        <v>1642</v>
-      </c>
     </row>
     <row r="11" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
@@ -6509,12 +6457,6 @@
       <c r="W11" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="Z11" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA11" s="18" t="s">
-        <v>1642</v>
-      </c>
     </row>
     <row r="12" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="s">
@@ -6586,12 +6528,6 @@
       <c r="W12" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="Z12" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA12" s="18" t="s">
-        <v>1642</v>
-      </c>
     </row>
     <row r="13" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="9" t="s">
@@ -6663,12 +6599,6 @@
       <c r="W13" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="Z13" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA13" s="18" t="s">
-        <v>1642</v>
-      </c>
     </row>
     <row r="14" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="9" t="s">
@@ -6740,12 +6670,6 @@
       <c r="W14" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="Z14" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA14" s="18" t="s">
-        <v>1642</v>
-      </c>
     </row>
     <row r="15" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="9" t="s">
@@ -6817,12 +6741,6 @@
       <c r="W15" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="Z15" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA15" s="18" t="s">
-        <v>1642</v>
-      </c>
     </row>
     <row r="16" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="9" t="s">
@@ -6894,12 +6812,6 @@
       <c r="W16" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="Z16" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA16" s="18" t="s">
-        <v>1642</v>
-      </c>
     </row>
     <row r="17" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="9" t="s">
@@ -6971,12 +6883,6 @@
       <c r="W17" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="Z17" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA17" s="18" t="s">
-        <v>1642</v>
-      </c>
     </row>
     <row r="18" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
@@ -7048,12 +6954,6 @@
       <c r="W18" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="Z18" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA18" s="18" t="s">
-        <v>1642</v>
-      </c>
     </row>
     <row r="19" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
@@ -7125,12 +7025,6 @@
       <c r="W19" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="Z19" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA19" s="18" t="s">
-        <v>1642</v>
-      </c>
     </row>
     <row r="20" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="6" t="s">
@@ -7202,9 +7096,6 @@
       <c r="W20" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AA20" s="18" t="s">
-        <v>1647</v>
-      </c>
     </row>
     <row r="21" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6" t="s">
@@ -7276,9 +7167,6 @@
       <c r="W21" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AA21" s="18" t="s">
-        <v>1647</v>
-      </c>
     </row>
     <row r="22" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="6" t="s">
@@ -7350,9 +7238,6 @@
       <c r="W22" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AA22" s="18" t="s">
-        <v>1647</v>
-      </c>
     </row>
     <row r="23" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="6" t="s">
@@ -7424,9 +7309,7 @@
       <c r="W23" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AA23" s="18" t="s">
-        <v>1647</v>
-      </c>
+      <c r="AA23" s="18"/>
     </row>
     <row r="24" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="6" t="s">
@@ -7498,9 +7381,7 @@
       <c r="W24" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AA24" s="18" t="s">
-        <v>1647</v>
-      </c>
+      <c r="AA24" s="18"/>
     </row>
     <row r="25" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="6" t="s">
@@ -7572,9 +7453,7 @@
       <c r="W25" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AA25" s="18" t="s">
-        <v>1647</v>
-      </c>
+      <c r="AA25" s="18"/>
     </row>
     <row r="26" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="6" t="s">
@@ -7646,9 +7525,6 @@
       <c r="W26" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AA26" s="18" t="s">
-        <v>1647</v>
-      </c>
     </row>
     <row r="27" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
@@ -7720,9 +7596,6 @@
       <c r="W27" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AA27" s="18" t="s">
-        <v>1647</v>
-      </c>
     </row>
     <row r="28" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
@@ -7794,9 +7667,6 @@
       <c r="W28" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AA28" s="18" t="s">
-        <v>1647</v>
-      </c>
     </row>
     <row r="29" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
@@ -7868,9 +7738,6 @@
       <c r="W29" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AA29" s="18" t="s">
-        <v>1647</v>
-      </c>
     </row>
     <row r="30" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
@@ -7942,9 +7809,6 @@
       <c r="W30" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AA30" s="18" t="s">
-        <v>1647</v>
-      </c>
     </row>
     <row r="31" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="5" t="s">
@@ -8016,9 +7880,6 @@
       <c r="W31" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AA31" s="18" t="s">
-        <v>1647</v>
-      </c>
     </row>
     <row r="32" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="8" t="s">
@@ -8090,11 +7951,8 @@
       <c r="W32" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AA32" s="18" t="s">
-        <v>1647</v>
-      </c>
-    </row>
-    <row r="33" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="33" spans="1:26" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
         <v>202</v>
       </c>
@@ -8164,11 +8022,8 @@
       <c r="W33" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AA33" s="18" t="s">
-        <v>1647</v>
-      </c>
-    </row>
-    <row r="34" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="34" spans="1:26" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="8" t="s">
         <v>205</v>
       </c>
@@ -8238,11 +8093,11 @@
       <c r="W34" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AA34" s="18" t="s">
-        <v>1647</v>
-      </c>
-    </row>
-    <row r="35" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="Z34" t="s">
+        <v>1643</v>
+      </c>
+    </row>
+    <row r="35" spans="1:26" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="5" t="s">
         <v>214</v>
       </c>
@@ -8312,11 +8167,11 @@
       <c r="W35" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AA35" s="18" t="s">
-        <v>1647</v>
-      </c>
-    </row>
-    <row r="36" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="Z35" t="s">
+        <v>1643</v>
+      </c>
+    </row>
+    <row r="36" spans="1:26" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="5" t="s">
         <v>217</v>
       </c>
@@ -8386,11 +8241,8 @@
       <c r="W36" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AA36" s="18" t="s">
-        <v>1647</v>
-      </c>
-    </row>
-    <row r="37" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="37" spans="1:26" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="6" t="s">
         <v>229</v>
       </c>
@@ -8460,11 +8312,8 @@
       <c r="W37" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AA37" s="18" t="s">
-        <v>1647</v>
-      </c>
-    </row>
-    <row r="38" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="38" spans="1:26" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="5" t="s">
         <v>233</v>
       </c>
@@ -8534,11 +8383,8 @@
       <c r="W38" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AA38" s="18" t="s">
-        <v>1647</v>
-      </c>
-    </row>
-    <row r="39" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="39" spans="1:26" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="5" t="s">
         <v>237</v>
       </c>
@@ -8602,11 +8448,8 @@
         <v>118</v>
       </c>
       <c r="W39" s="5"/>
-      <c r="AA39" s="18" t="s">
-        <v>1647</v>
-      </c>
-    </row>
-    <row r="40" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="40" spans="1:26" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="5" t="s">
         <v>251</v>
       </c>
@@ -8670,11 +8513,8 @@
         <v>118</v>
       </c>
       <c r="W40" s="5"/>
-      <c r="AA40" s="18" t="s">
-        <v>1647</v>
-      </c>
-    </row>
-    <row r="41" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="41" spans="1:26" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="5" t="s">
         <v>253</v>
       </c>
@@ -8738,14 +8578,8 @@
         <v>41</v>
       </c>
       <c r="W41" s="5"/>
-      <c r="Z41" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA41" s="18" t="s">
-        <v>1642</v>
-      </c>
-    </row>
-    <row r="42" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="42" spans="1:26" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="5" t="s">
         <v>260</v>
       </c>
@@ -8809,11 +8643,8 @@
         <v>118</v>
       </c>
       <c r="W42" s="5"/>
-      <c r="AA42" s="18" t="s">
-        <v>1647</v>
-      </c>
-    </row>
-    <row r="43" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="43" spans="1:26" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="5" t="s">
         <v>268</v>
       </c>
@@ -8877,11 +8708,8 @@
         <v>55</v>
       </c>
       <c r="W43" s="5"/>
-      <c r="AA43" s="18" t="s">
-        <v>1647</v>
-      </c>
-    </row>
-    <row r="44" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="44" spans="1:26" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="5" t="s">
         <v>272</v>
       </c>
@@ -8945,11 +8773,8 @@
         <v>55</v>
       </c>
       <c r="W44" s="5"/>
-      <c r="AA44" s="18" t="s">
-        <v>1647</v>
-      </c>
-    </row>
-    <row r="45" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="45" spans="1:26" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="5" t="s">
         <v>275</v>
       </c>
@@ -9013,11 +8838,8 @@
         <v>41</v>
       </c>
       <c r="W45" s="5"/>
-      <c r="AA45" s="18" t="s">
-        <v>1647</v>
-      </c>
-    </row>
-    <row r="46" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="46" spans="1:26" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="5" t="s">
         <v>276</v>
       </c>
@@ -9081,11 +8903,8 @@
         <v>41</v>
       </c>
       <c r="W46" s="5"/>
-      <c r="AA46" s="18" t="s">
-        <v>1647</v>
-      </c>
-    </row>
-    <row r="47" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="47" spans="1:26" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="5" t="s">
         <v>280</v>
       </c>
@@ -9155,11 +8974,8 @@
       <c r="W47" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="AA47" s="18" t="s">
-        <v>1647</v>
-      </c>
-    </row>
-    <row r="48" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="48" spans="1:26" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="5" t="s">
         <v>280</v>
       </c>
@@ -9229,11 +9045,8 @@
       <c r="W48" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="AA48" s="18" t="s">
-        <v>1647</v>
-      </c>
-    </row>
-    <row r="49" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="49" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="5" t="s">
         <v>292</v>
       </c>
@@ -9303,11 +9116,8 @@
       <c r="W49" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="AA49" s="18" t="s">
-        <v>1647</v>
-      </c>
-    </row>
-    <row r="50" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="50" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="5" t="s">
         <v>297</v>
       </c>
@@ -9377,14 +9187,8 @@
       <c r="W50" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="Z50" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA50" s="18" t="s">
-        <v>1642</v>
-      </c>
-    </row>
-    <row r="51" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="51" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="9" t="s">
         <v>305</v>
       </c>
@@ -9452,11 +9256,8 @@
       <c r="W51" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AA51" s="18" t="s">
-        <v>1647</v>
-      </c>
-    </row>
-    <row r="52" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="52" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="9" t="s">
         <v>310</v>
       </c>
@@ -9526,11 +9327,8 @@
       <c r="W52" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="AA52" s="18" t="s">
-        <v>1647</v>
-      </c>
-    </row>
-    <row r="53" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="53" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="9" t="s">
         <v>310</v>
       </c>
@@ -9600,11 +9398,8 @@
       <c r="W53" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="AA53" s="18" t="s">
-        <v>1647</v>
-      </c>
-    </row>
-    <row r="54" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="54" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="9" t="s">
         <v>316</v>
       </c>
@@ -9672,11 +9467,8 @@
       <c r="W54" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="AA54" s="18" t="s">
-        <v>1647</v>
-      </c>
-    </row>
-    <row r="55" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="55" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="9" t="s">
         <v>321</v>
       </c>
@@ -9744,11 +9536,8 @@
       <c r="W55" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="AA55" s="18" t="s">
-        <v>1647</v>
-      </c>
-    </row>
-    <row r="56" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="56" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="9" t="s">
         <v>324</v>
       </c>
@@ -9816,11 +9605,8 @@
       <c r="W56" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AA56" s="18" t="s">
-        <v>1647</v>
-      </c>
-    </row>
-    <row r="57" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="57" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="9" t="s">
         <v>327</v>
       </c>
@@ -9888,11 +9674,8 @@
       <c r="W57" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AA57" s="18" t="s">
-        <v>1647</v>
-      </c>
-    </row>
-    <row r="58" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="58" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="9" t="s">
         <v>329</v>
       </c>
@@ -9960,11 +9743,8 @@
       <c r="W58" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AA58" s="18" t="s">
-        <v>1647</v>
-      </c>
-    </row>
-    <row r="59" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="59" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="9" t="s">
         <v>334</v>
       </c>
@@ -10032,11 +9812,8 @@
       <c r="W59" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AA59" s="18" t="s">
-        <v>1647</v>
-      </c>
-    </row>
-    <row r="60" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="60" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="9" t="s">
         <v>338</v>
       </c>
@@ -10104,11 +9881,8 @@
       <c r="W60" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AA60" s="18" t="s">
-        <v>1647</v>
-      </c>
-    </row>
-    <row r="61" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="61" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="9" t="s">
         <v>340</v>
       </c>
@@ -10176,11 +9950,8 @@
       <c r="W61" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AA61" s="18" t="s">
-        <v>1647</v>
-      </c>
-    </row>
-    <row r="62" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="62" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="9" t="s">
         <v>341</v>
       </c>
@@ -10248,11 +10019,8 @@
       <c r="W62" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AA62" s="18" t="s">
-        <v>1647</v>
-      </c>
-    </row>
-    <row r="63" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="63" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="9" t="s">
         <v>343</v>
       </c>
@@ -10320,11 +10088,8 @@
       <c r="W63" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AA63" s="18" t="s">
-        <v>1647</v>
-      </c>
-    </row>
-    <row r="64" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="64" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="9" t="s">
         <v>347</v>
       </c>
@@ -10392,9 +10157,6 @@
       <c r="W64" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AA64" s="18" t="s">
-        <v>1647</v>
-      </c>
     </row>
     <row r="65" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="5" t="s">
@@ -10464,9 +10226,6 @@
       <c r="W65" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AA65" s="18" t="s">
-        <v>1647</v>
-      </c>
     </row>
     <row r="66" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="5" t="s">
@@ -10538,9 +10297,6 @@
       <c r="W66" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AA66" s="18" t="s">
-        <v>1647</v>
-      </c>
     </row>
     <row r="67" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="5" t="s">
@@ -10612,9 +10368,6 @@
       <c r="W67" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AA67" s="18" t="s">
-        <v>1647</v>
-      </c>
     </row>
     <row r="68" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="5" t="s">
@@ -10680,8 +10433,8 @@
         <v>118</v>
       </c>
       <c r="W68" s="5"/>
-      <c r="AA68" s="18" t="s">
-        <v>1647</v>
+      <c r="Z68" t="s">
+        <v>1643</v>
       </c>
     </row>
     <row r="69" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -10748,12 +10501,6 @@
         <v>118</v>
       </c>
       <c r="W69" s="5"/>
-      <c r="Z69" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA69" s="18" t="s">
-        <v>1642</v>
-      </c>
     </row>
     <row r="70" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="5" t="s">
@@ -10819,9 +10566,6 @@
         <v>149</v>
       </c>
       <c r="W70" s="5"/>
-      <c r="AA70" s="18" t="s">
-        <v>1642</v>
-      </c>
     </row>
     <row r="71" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="5" t="s">
@@ -10887,9 +10631,6 @@
         <v>149</v>
       </c>
       <c r="W71" s="5"/>
-      <c r="AA71" s="18" t="s">
-        <v>1642</v>
-      </c>
     </row>
     <row r="72" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="5" t="s">
@@ -10961,9 +10702,6 @@
       <c r="W72" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="AA72" s="18" t="s">
-        <v>1642</v>
-      </c>
     </row>
     <row r="73" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="5" t="s">
@@ -11035,9 +10773,6 @@
       <c r="W73" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="AA73" s="18" t="s">
-        <v>1642</v>
-      </c>
     </row>
     <row r="74" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="5" t="s">
@@ -11109,9 +10844,6 @@
       <c r="W74" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="AA74" s="18" t="s">
-        <v>1642</v>
-      </c>
     </row>
     <row r="75" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="5" t="s">
@@ -11181,9 +10913,6 @@
         <v>91</v>
       </c>
       <c r="W75" s="5"/>
-      <c r="AA75" s="18" t="s">
-        <v>1642</v>
-      </c>
     </row>
     <row r="76" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="5" t="s">
@@ -11253,9 +10982,6 @@
         <v>91</v>
       </c>
       <c r="W76" s="5"/>
-      <c r="AA76" s="18" t="s">
-        <v>1642</v>
-      </c>
     </row>
     <row r="77" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" s="5" t="s">
@@ -11321,9 +11047,6 @@
         <v>41</v>
       </c>
       <c r="W77" s="5"/>
-      <c r="AA77" s="18" t="s">
-        <v>1642</v>
-      </c>
     </row>
     <row r="78" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" s="5" t="s">
@@ -11389,9 +11112,6 @@
         <v>41</v>
       </c>
       <c r="W78" s="5"/>
-      <c r="AA78" s="18" t="s">
-        <v>1642</v>
-      </c>
     </row>
     <row r="79" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="5" t="s">
@@ -11461,8 +11181,8 @@
         <v>41</v>
       </c>
       <c r="W79" s="5"/>
-      <c r="AA79" s="18" t="s">
-        <v>1642</v>
+      <c r="AA79" t="s">
+        <v>1643</v>
       </c>
     </row>
     <row r="80" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -11533,8 +11253,8 @@
         <v>41</v>
       </c>
       <c r="W80" s="5"/>
-      <c r="AA80" s="18" t="s">
-        <v>1642</v>
+      <c r="AA80" t="s">
+        <v>1643</v>
       </c>
     </row>
     <row r="81" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -11607,9 +11327,7 @@
       <c r="W81" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AA81" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA81"/>
     </row>
     <row r="82" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="9" t="s">
@@ -11681,9 +11399,7 @@
       <c r="W82" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AA82" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA82"/>
     </row>
     <row r="83" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A83" s="9" t="s">
@@ -11755,9 +11471,7 @@
       <c r="W83" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AA83" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA83"/>
     </row>
     <row r="84" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A84" s="9" t="s">
@@ -11829,9 +11543,7 @@
       <c r="W84" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AA84" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA84"/>
     </row>
     <row r="85" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A85" s="9" t="s">
@@ -11901,9 +11613,7 @@
       <c r="W85" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AA85" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA85"/>
     </row>
     <row r="86" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A86" s="9" t="s">
@@ -11973,9 +11683,7 @@
       <c r="W86" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="AA86" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA86"/>
     </row>
     <row r="87" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A87" s="9" t="s">
@@ -12045,9 +11753,7 @@
       <c r="W87" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="AA87" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA87"/>
     </row>
     <row r="88" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A88" s="9" t="s">
@@ -12119,9 +11825,7 @@
       <c r="W88" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="AA88" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA88"/>
     </row>
     <row r="89" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A89" s="9" t="s">
@@ -12189,9 +11893,7 @@
         <v>41</v>
       </c>
       <c r="W89" s="5"/>
-      <c r="AA89" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA89"/>
     </row>
     <row r="90" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" s="9" t="s">
@@ -12261,9 +11963,7 @@
         <v>55</v>
       </c>
       <c r="W90" s="5"/>
-      <c r="AA90" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA90"/>
     </row>
     <row r="91" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A91" s="9" t="s">
@@ -12335,9 +12035,7 @@
       <c r="W91" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="AA91" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA91"/>
     </row>
     <row r="92" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A92" s="9" t="s">
@@ -12409,9 +12107,7 @@
       <c r="W92" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="AA92" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA92"/>
     </row>
     <row r="93" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A93" s="9" t="s">
@@ -12483,9 +12179,7 @@
       <c r="W93" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="AA93" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA93"/>
     </row>
     <row r="94" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" s="9" t="s">
@@ -12555,9 +12249,7 @@
       <c r="W94" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="AA94" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA94"/>
     </row>
     <row r="95" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A95" s="9" t="s">
@@ -12629,9 +12321,7 @@
       <c r="W95" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="AA95" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA95"/>
     </row>
     <row r="96" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A96" s="9" t="s">
@@ -12703,9 +12393,7 @@
       <c r="W96" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="AA96" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA96"/>
     </row>
     <row r="97" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A97" s="9" t="s">
@@ -12777,9 +12465,7 @@
       <c r="W97" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="AA97" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA97"/>
     </row>
     <row r="98" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" s="9" t="s">
@@ -12851,9 +12537,7 @@
       <c r="W98" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="AA98" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA98"/>
     </row>
     <row r="99" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A99" s="9" t="s">
@@ -12921,9 +12605,7 @@
         <v>41</v>
       </c>
       <c r="W99" s="5"/>
-      <c r="AA99" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA99"/>
     </row>
     <row r="100" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A100" s="9" t="s">
@@ -12991,9 +12673,7 @@
         <v>41</v>
       </c>
       <c r="W100" s="5"/>
-      <c r="AA100" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA100"/>
     </row>
     <row r="101" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A101" s="5" t="s">
@@ -13063,9 +12743,7 @@
         <v>91</v>
       </c>
       <c r="W101" s="5"/>
-      <c r="AA101" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA101"/>
     </row>
     <row r="102" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A102" s="5" t="s">
@@ -13131,9 +12809,7 @@
         <v>149</v>
       </c>
       <c r="W102" s="5"/>
-      <c r="AA102" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA102"/>
     </row>
     <row r="103" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A103" s="9" t="s">
@@ -13205,8 +12881,8 @@
       <c r="W103" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="AA103" s="18" t="s">
-        <v>1642</v>
+      <c r="AA103" t="s">
+        <v>1643</v>
       </c>
     </row>
     <row r="104" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -13279,8 +12955,8 @@
       <c r="W104" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="AA104" s="18" t="s">
-        <v>1642</v>
+      <c r="AA104" t="s">
+        <v>1643</v>
       </c>
     </row>
     <row r="105" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -13353,9 +13029,7 @@
       <c r="W105" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="AA105" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA105"/>
     </row>
     <row r="106" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A106" s="9" t="s">
@@ -13427,9 +13101,7 @@
       <c r="W106" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="AA106" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA106"/>
     </row>
     <row r="107" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A107" s="9" t="s">
@@ -13501,9 +13173,7 @@
       <c r="W107" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="AA107" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA107"/>
     </row>
     <row r="108" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A108" s="9" t="s">
@@ -13575,9 +13245,7 @@
       <c r="W108" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="AA108" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA108"/>
     </row>
     <row r="109" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A109" s="9" t="s">
@@ -13649,8 +13317,8 @@
       <c r="W109" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="AA109" s="18" t="s">
-        <v>1642</v>
+      <c r="AA109" t="s">
+        <v>1643</v>
       </c>
     </row>
     <row r="110" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -13723,8 +13391,8 @@
       <c r="W110" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="AA110" s="18" t="s">
-        <v>1642</v>
+      <c r="AA110" t="s">
+        <v>1643</v>
       </c>
     </row>
     <row r="111" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -13797,9 +13465,7 @@
       <c r="W111" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="AA111" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA111"/>
     </row>
     <row r="112" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A112" s="9" t="s">
@@ -13871,9 +13537,7 @@
       <c r="W112" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="AA112" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA112"/>
     </row>
     <row r="113" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A113" s="9" t="s">
@@ -13945,9 +13609,7 @@
       <c r="W113" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="AA113" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA113"/>
     </row>
     <row r="114" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A114" s="9" t="s">
@@ -14019,9 +13681,7 @@
       <c r="W114" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="AA114" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA114"/>
     </row>
     <row r="115" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A115" s="9" t="s">
@@ -14093,9 +13753,7 @@
       <c r="W115" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="AA115" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA115"/>
     </row>
     <row r="116" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A116" s="9" t="s">
@@ -14167,9 +13825,7 @@
       <c r="W116" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="AA116" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA116"/>
     </row>
     <row r="117" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A117" s="9" t="s">
@@ -14241,9 +13897,7 @@
       <c r="W117" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="AA117" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA117"/>
     </row>
     <row r="118" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A118" s="9" t="s">
@@ -14315,9 +13969,7 @@
       <c r="W118" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="AA118" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA118"/>
     </row>
     <row r="119" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A119" s="9" t="s">
@@ -14389,9 +14041,7 @@
       <c r="W119" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="AA119" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA119"/>
     </row>
     <row r="120" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A120" s="9" t="s">
@@ -14463,9 +14113,7 @@
       <c r="W120" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="AA120" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA120"/>
     </row>
     <row r="121" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A121" s="9" t="s">
@@ -14537,9 +14185,7 @@
       <c r="W121" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="AA121" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA121"/>
     </row>
     <row r="122" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A122" s="9" t="s">
@@ -14611,9 +14257,7 @@
       <c r="W122" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="AA122" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA122"/>
     </row>
     <row r="123" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A123" s="9" t="s">
@@ -14685,9 +14329,7 @@
       <c r="W123" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="AA123" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA123"/>
     </row>
     <row r="124" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A124" s="9" t="s">
@@ -14759,9 +14401,7 @@
       <c r="W124" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="AA124" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA124"/>
     </row>
     <row r="125" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A125" s="9" t="s">
@@ -14833,9 +14473,7 @@
       <c r="W125" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="AA125" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA125"/>
     </row>
     <row r="126" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A126" s="9" t="s">
@@ -14907,9 +14545,7 @@
       <c r="W126" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="AA126" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA126"/>
     </row>
     <row r="127" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A127" s="9" t="s">
@@ -14981,9 +14617,7 @@
       <c r="W127" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="AA127" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA127"/>
     </row>
     <row r="128" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A128" s="9" t="s">
@@ -15055,9 +14689,7 @@
       <c r="W128" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="AA128" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA128"/>
     </row>
     <row r="129" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A129" s="9" t="s">
@@ -15129,9 +14761,7 @@
       <c r="W129" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="AA129" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA129"/>
     </row>
     <row r="130" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A130" s="9" t="s">
@@ -15203,9 +14833,7 @@
       <c r="W130" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="AA130" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA130"/>
     </row>
     <row r="131" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A131" s="9" t="s">
@@ -15277,9 +14905,7 @@
       <c r="W131" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="AA131" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA131"/>
     </row>
     <row r="132" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A132" s="9" t="s">
@@ -15351,9 +14977,7 @@
       <c r="W132" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="AA132" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA132"/>
     </row>
     <row r="133" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A133" s="9" t="s">
@@ -15423,9 +15047,7 @@
         <v>91</v>
       </c>
       <c r="W133" s="5"/>
-      <c r="AA133" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA133"/>
     </row>
     <row r="134" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A134" s="11" t="s">
@@ -15493,8 +15115,8 @@
         <v>91</v>
       </c>
       <c r="W134" s="12"/>
-      <c r="AA134" s="18" t="s">
-        <v>1642</v>
+      <c r="AA134" t="s">
+        <v>1643</v>
       </c>
     </row>
     <row r="135" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -15561,9 +15183,7 @@
         <v>118</v>
       </c>
       <c r="W135" s="10"/>
-      <c r="AA135" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA135"/>
     </row>
     <row r="136" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A136" s="10" t="s">
@@ -15629,8 +15249,8 @@
         <v>149</v>
       </c>
       <c r="W136" s="10"/>
-      <c r="AA136" s="18" t="s">
-        <v>1642</v>
+      <c r="AA136" t="s">
+        <v>1644</v>
       </c>
     </row>
     <row r="137" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -15697,8 +15317,8 @@
         <v>149</v>
       </c>
       <c r="W137" s="10"/>
-      <c r="AA137" s="18" t="s">
-        <v>1642</v>
+      <c r="AA137" t="s">
+        <v>1644</v>
       </c>
     </row>
     <row r="138" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -15765,9 +15385,7 @@
         <v>55</v>
       </c>
       <c r="W138" s="10"/>
-      <c r="AA138" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA138"/>
     </row>
     <row r="139" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A139" s="10" t="s">
@@ -15827,9 +15445,10 @@
         <v>55</v>
       </c>
       <c r="W139" s="10"/>
-      <c r="AA139" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="Z139" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA139"/>
     </row>
     <row r="140" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A140" s="10" t="s">
@@ -15889,9 +15508,10 @@
         <v>55</v>
       </c>
       <c r="W140" s="10"/>
-      <c r="AA140" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="Z140" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA140"/>
     </row>
     <row r="141" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A141" s="10" t="s">
@@ -15951,9 +15571,10 @@
         <v>55</v>
       </c>
       <c r="W141" s="10"/>
-      <c r="AA141" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="Z141" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA141"/>
     </row>
     <row r="142" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A142" s="10" t="s">
@@ -16013,9 +15634,10 @@
         <v>55</v>
       </c>
       <c r="W142" s="10"/>
-      <c r="AA142" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="Z142" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA142"/>
     </row>
     <row r="143" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A143" s="10" t="s">
@@ -16075,9 +15697,10 @@
         <v>55</v>
       </c>
       <c r="W143" s="10"/>
-      <c r="AA143" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="Z143" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA143"/>
     </row>
     <row r="144" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A144" s="10" t="s">
@@ -16137,9 +15760,10 @@
         <v>55</v>
       </c>
       <c r="W144" s="10"/>
-      <c r="AA144" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="Z144" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA144"/>
     </row>
     <row r="145" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A145" s="10" t="s">
@@ -16199,9 +15823,10 @@
         <v>55</v>
       </c>
       <c r="W145" s="10"/>
-      <c r="AA145" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="Z145" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA145"/>
     </row>
     <row r="146" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A146" s="10" t="s">
@@ -16261,9 +15886,10 @@
         <v>55</v>
       </c>
       <c r="W146" s="10"/>
-      <c r="AA146" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="Z146" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA146"/>
     </row>
     <row r="147" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A147" s="10" t="s">
@@ -16323,9 +15949,10 @@
         <v>55</v>
       </c>
       <c r="W147" s="10"/>
-      <c r="AA147" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="Z147" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA147"/>
     </row>
     <row r="148" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A148" s="10" t="s">
@@ -16385,9 +16012,10 @@
         <v>55</v>
       </c>
       <c r="W148" s="10"/>
-      <c r="AA148" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="Z148" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA148"/>
     </row>
     <row r="149" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A149" s="10" t="s">
@@ -16447,9 +16075,10 @@
         <v>55</v>
       </c>
       <c r="W149" s="10"/>
-      <c r="AA149" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="Z149" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA149"/>
     </row>
     <row r="150" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A150" s="10" t="s">
@@ -16509,9 +16138,10 @@
         <v>55</v>
       </c>
       <c r="W150" s="10"/>
-      <c r="AA150" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="Z150" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA150"/>
     </row>
     <row r="151" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A151" s="10" t="s">
@@ -16571,9 +16201,10 @@
         <v>55</v>
       </c>
       <c r="W151" s="10"/>
-      <c r="AA151" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="Z151" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA151"/>
     </row>
     <row r="152" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A152" s="10" t="s">
@@ -16633,9 +16264,10 @@
         <v>55</v>
       </c>
       <c r="W152" s="10"/>
-      <c r="AA152" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="Z152" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA152"/>
     </row>
     <row r="153" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A153" s="10" t="s">
@@ -16695,9 +16327,10 @@
         <v>55</v>
       </c>
       <c r="W153" s="10"/>
-      <c r="AA153" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="Z153" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA153"/>
     </row>
     <row r="154" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A154" s="10" t="s">
@@ -16757,9 +16390,10 @@
         <v>55</v>
       </c>
       <c r="W154" s="10"/>
-      <c r="AA154" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="Z154" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA154"/>
     </row>
     <row r="155" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A155" s="10" t="s">
@@ -16819,9 +16453,10 @@
         <v>55</v>
       </c>
       <c r="W155" s="10"/>
-      <c r="AA155" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="Z155" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA155"/>
     </row>
     <row r="156" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A156" s="10" t="s">
@@ -16881,9 +16516,10 @@
         <v>55</v>
       </c>
       <c r="W156" s="10"/>
-      <c r="AA156" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="Z156" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA156"/>
     </row>
     <row r="157" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A157" s="10" t="s">
@@ -16943,9 +16579,10 @@
         <v>55</v>
       </c>
       <c r="W157" s="10"/>
-      <c r="AA157" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="Z157" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA157"/>
     </row>
     <row r="158" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A158" s="10" t="s">
@@ -17011,9 +16648,10 @@
         <v>55</v>
       </c>
       <c r="W158" s="10"/>
-      <c r="AA158" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="Z158" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA158"/>
     </row>
     <row r="159" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A159" s="10" t="s">
@@ -17073,9 +16711,10 @@
         <v>55</v>
       </c>
       <c r="W159" s="10"/>
-      <c r="AA159" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="Z159" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA159"/>
     </row>
     <row r="160" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A160" s="10" t="s">
@@ -17135,9 +16774,10 @@
         <v>55</v>
       </c>
       <c r="W160" s="10"/>
-      <c r="AA160" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="Z160" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA160"/>
     </row>
     <row r="161" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A161" s="10" t="s">
@@ -17197,9 +16837,10 @@
         <v>55</v>
       </c>
       <c r="W161" s="10"/>
-      <c r="AA161" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="Z161" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA161"/>
     </row>
     <row r="162" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A162" s="10" t="s">
@@ -17259,9 +16900,10 @@
         <v>55</v>
       </c>
       <c r="W162" s="10"/>
-      <c r="AA162" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="Z162" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA162"/>
     </row>
     <row r="163" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A163" s="10" t="s">
@@ -17321,9 +16963,10 @@
         <v>55</v>
       </c>
       <c r="W163" s="10"/>
-      <c r="AA163" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="Z163" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA163"/>
     </row>
     <row r="164" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A164" s="10" t="s">
@@ -17383,9 +17026,10 @@
         <v>55</v>
       </c>
       <c r="W164" s="10"/>
-      <c r="AA164" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="Z164" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA164"/>
     </row>
     <row r="165" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A165" s="10" t="s">
@@ -17445,9 +17089,10 @@
         <v>55</v>
       </c>
       <c r="W165" s="10"/>
-      <c r="AA165" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="Z165" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA165"/>
     </row>
     <row r="166" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A166" s="10" t="s">
@@ -17507,9 +17152,10 @@
         <v>55</v>
       </c>
       <c r="W166" s="10"/>
-      <c r="AA166" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="Z166" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA166"/>
     </row>
     <row r="167" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A167" s="10" t="s">
@@ -17575,9 +17221,7 @@
         <v>41</v>
       </c>
       <c r="W167" s="10"/>
-      <c r="AA167" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA167"/>
     </row>
     <row r="168" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A168" s="10" t="s">
@@ -17643,9 +17287,7 @@
         <v>55</v>
       </c>
       <c r="W168" s="10"/>
-      <c r="AA168" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA168"/>
     </row>
     <row r="169" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A169" s="10" t="s">
@@ -17711,9 +17353,7 @@
         <v>55</v>
       </c>
       <c r="W169" s="10"/>
-      <c r="AA169" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA169"/>
     </row>
     <row r="170" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A170" s="10" t="s">
@@ -17779,9 +17419,7 @@
         <v>55</v>
       </c>
       <c r="W170" s="10"/>
-      <c r="AA170" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA170"/>
     </row>
     <row r="171" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A171" s="10" t="s">
@@ -17847,9 +17485,10 @@
         <v>166</v>
       </c>
       <c r="W171" s="10"/>
-      <c r="AA171" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="Z171" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA171"/>
     </row>
     <row r="172" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A172" s="10" t="s">
@@ -17915,9 +17554,7 @@
         <v>41</v>
       </c>
       <c r="W172" s="10"/>
-      <c r="AA172" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA172"/>
     </row>
     <row r="173" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A173" s="10" t="s">
@@ -17983,9 +17620,7 @@
         <v>41</v>
       </c>
       <c r="W173" s="10"/>
-      <c r="AA173" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA173"/>
     </row>
     <row r="174" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A174" s="10" t="s">
@@ -18051,9 +17686,7 @@
         <v>41</v>
       </c>
       <c r="W174" s="10"/>
-      <c r="AA174" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA174"/>
     </row>
     <row r="175" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A175" s="15" t="s">
@@ -18119,12 +17752,7 @@
         <v>149</v>
       </c>
       <c r="W175" s="15"/>
-      <c r="Z175" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA175" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA175"/>
     </row>
     <row r="176" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A176" s="10" t="s">
@@ -18190,9 +17818,7 @@
         <v>149</v>
       </c>
       <c r="W176" s="10"/>
-      <c r="AA176" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA176"/>
     </row>
     <row r="177" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A177" s="10" t="s">
@@ -18260,9 +17886,7 @@
         <v>149</v>
       </c>
       <c r="W177" s="10"/>
-      <c r="AA177" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA177"/>
     </row>
     <row r="178" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A178" s="10" t="s">
@@ -18326,12 +17950,7 @@
         <v>149</v>
       </c>
       <c r="W178" s="10"/>
-      <c r="Z178" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA178" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA178"/>
     </row>
     <row r="179" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A179" s="10" t="s">
@@ -18397,9 +18016,7 @@
         <v>149</v>
       </c>
       <c r="W179" s="10"/>
-      <c r="AA179" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA179"/>
     </row>
     <row r="180" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A180" s="10" t="s">
@@ -18467,12 +18084,7 @@
         <v>149</v>
       </c>
       <c r="W180" s="10"/>
-      <c r="Z180" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA180" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA180"/>
     </row>
     <row r="181" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A181" s="10" t="s">
@@ -18540,9 +18152,7 @@
         <v>149</v>
       </c>
       <c r="W181" s="10"/>
-      <c r="AA181" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA181"/>
     </row>
     <row r="182" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A182" s="10" t="s">
@@ -18610,9 +18220,7 @@
         <v>149</v>
       </c>
       <c r="W182" s="10"/>
-      <c r="AA182" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA182"/>
     </row>
     <row r="183" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A183" s="10" t="s">
@@ -18680,9 +18288,7 @@
         <v>149</v>
       </c>
       <c r="W183" s="10"/>
-      <c r="AA183" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA183"/>
     </row>
     <row r="184" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A184" s="10" t="s">
@@ -18750,9 +18356,7 @@
         <v>41</v>
       </c>
       <c r="W184" s="10"/>
-      <c r="AA184" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA184"/>
     </row>
     <row r="185" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A185" s="10" t="s">
@@ -18820,8 +18424,8 @@
         <v>91</v>
       </c>
       <c r="W185" s="10"/>
-      <c r="AA185" s="18" t="s">
-        <v>1642</v>
+      <c r="AA185" t="s">
+        <v>1643</v>
       </c>
     </row>
     <row r="186" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -18890,9 +18494,7 @@
         <v>91</v>
       </c>
       <c r="W186" s="10"/>
-      <c r="AA186" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA186"/>
     </row>
     <row r="187" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A187" s="10" t="s">
@@ -18960,9 +18562,7 @@
         <v>91</v>
       </c>
       <c r="W187" s="10"/>
-      <c r="AA187" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA187"/>
     </row>
     <row r="188" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A188" s="10" t="s">
@@ -19030,9 +18630,7 @@
         <v>91</v>
       </c>
       <c r="W188" s="10"/>
-      <c r="AA188" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA188"/>
     </row>
     <row r="189" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A189" s="10" t="s">
@@ -19100,9 +18698,7 @@
         <v>91</v>
       </c>
       <c r="W189" s="10"/>
-      <c r="AA189" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA189"/>
     </row>
     <row r="190" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A190" s="10" t="s">
@@ -19170,9 +18766,7 @@
         <v>91</v>
       </c>
       <c r="W190" s="10"/>
-      <c r="AA190" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA190"/>
     </row>
     <row r="191" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A191" s="10" t="s">
@@ -19240,9 +18834,7 @@
         <v>91</v>
       </c>
       <c r="W191" s="10"/>
-      <c r="AA191" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA191"/>
     </row>
     <row r="192" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A192" s="10" t="s">
@@ -19310,9 +18902,7 @@
         <v>91</v>
       </c>
       <c r="W192" s="10"/>
-      <c r="AA192" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA192"/>
     </row>
     <row r="193" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A193" s="10" t="s">
@@ -19380,8 +18970,8 @@
         <v>91</v>
       </c>
       <c r="W193" s="10"/>
-      <c r="AA193" s="18" t="s">
-        <v>1642</v>
+      <c r="AA193" t="s">
+        <v>1644</v>
       </c>
     </row>
     <row r="194" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -19450,12 +19040,7 @@
         <v>91</v>
       </c>
       <c r="W194" s="10"/>
-      <c r="Z194" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA194" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA194"/>
     </row>
     <row r="195" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A195" s="10" t="s">
@@ -19521,12 +19106,7 @@
         <v>91</v>
       </c>
       <c r="W195" s="10"/>
-      <c r="Z195" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA195" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA195"/>
     </row>
     <row r="196" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A196" s="10" t="s">
@@ -19592,12 +19172,7 @@
         <v>91</v>
       </c>
       <c r="W196" s="10"/>
-      <c r="Z196" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA196" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA196"/>
     </row>
     <row r="197" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A197" s="10" t="s">
@@ -19665,9 +19240,10 @@
         <v>91</v>
       </c>
       <c r="W197" s="10"/>
-      <c r="AA197" s="18" t="s">
-        <v>1647</v>
-      </c>
+      <c r="Z197" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA197"/>
     </row>
     <row r="198" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A198" s="10" t="s">
@@ -19735,9 +19311,10 @@
         <v>91</v>
       </c>
       <c r="W198" s="10"/>
-      <c r="AA198" s="18" t="s">
-        <v>1647</v>
-      </c>
+      <c r="Z198" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA198"/>
     </row>
     <row r="199" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A199" s="10" t="s">
@@ -19805,9 +19382,10 @@
         <v>91</v>
       </c>
       <c r="W199" s="10"/>
-      <c r="AA199" s="18" t="s">
-        <v>1647</v>
-      </c>
+      <c r="Z199" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA199"/>
     </row>
     <row r="200" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A200" s="10" t="s">
@@ -19871,9 +19449,10 @@
         <v>91</v>
       </c>
       <c r="W200" s="10"/>
-      <c r="AA200" s="18" t="s">
-        <v>1647</v>
-      </c>
+      <c r="Z200" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA200"/>
     </row>
     <row r="201" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A201" s="10" t="s">
@@ -19941,9 +19520,10 @@
         <v>91</v>
       </c>
       <c r="W201" s="10"/>
-      <c r="AA201" s="18" t="s">
-        <v>1647</v>
-      </c>
+      <c r="Z201" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA201"/>
     </row>
     <row r="202" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A202" s="10" t="s">
@@ -20011,9 +19591,7 @@
         <v>149</v>
       </c>
       <c r="W202" s="10"/>
-      <c r="AA202" s="18" t="s">
-        <v>1647</v>
-      </c>
+      <c r="AA202"/>
     </row>
     <row r="203" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A203" s="10" t="s">
@@ -20081,12 +19659,7 @@
         <v>149</v>
       </c>
       <c r="W203" s="10"/>
-      <c r="Z203" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA203" s="18" t="s">
-        <v>1647</v>
-      </c>
+      <c r="AA203"/>
     </row>
     <row r="204" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A204" s="10" t="s">
@@ -20154,9 +19727,7 @@
         <v>149</v>
       </c>
       <c r="W204" s="10"/>
-      <c r="AA204" s="18" t="s">
-        <v>1647</v>
-      </c>
+      <c r="AA204"/>
     </row>
     <row r="205" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A205" s="10" t="s">
@@ -20224,9 +19795,7 @@
         <v>149</v>
       </c>
       <c r="W205" s="10"/>
-      <c r="AA205" s="18" t="s">
-        <v>1647</v>
-      </c>
+      <c r="AA205"/>
     </row>
     <row r="206" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A206" s="10" t="s">
@@ -20294,12 +19863,7 @@
         <v>149</v>
       </c>
       <c r="W206" s="10"/>
-      <c r="Z206" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA206" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA206"/>
     </row>
     <row r="207" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A207" s="10" t="s">
@@ -20367,9 +19931,7 @@
         <v>149</v>
       </c>
       <c r="W207" s="10"/>
-      <c r="AA207" s="18" t="s">
-        <v>1647</v>
-      </c>
+      <c r="AA207"/>
     </row>
     <row r="208" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A208" s="10" t="s">
@@ -20437,9 +19999,7 @@
         <v>91</v>
       </c>
       <c r="W208" s="10"/>
-      <c r="AA208" s="18" t="s">
-        <v>1647</v>
-      </c>
+      <c r="AA208"/>
     </row>
     <row r="209" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A209" s="10" t="s">
@@ -20507,9 +20067,7 @@
         <v>55</v>
       </c>
       <c r="W209" s="10"/>
-      <c r="AA209" s="18" t="s">
-        <v>1647</v>
-      </c>
+      <c r="AA209"/>
     </row>
     <row r="210" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A210" s="10" t="s">
@@ -20577,9 +20135,7 @@
         <v>41</v>
       </c>
       <c r="W210" s="10"/>
-      <c r="AA210" s="18" t="s">
-        <v>1647</v>
-      </c>
+      <c r="AA210"/>
     </row>
     <row r="211" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A211" s="10" t="s">
@@ -20647,9 +20203,7 @@
         <v>41</v>
       </c>
       <c r="W211" s="10"/>
-      <c r="AA211" s="18" t="s">
-        <v>1647</v>
-      </c>
+      <c r="AA211"/>
     </row>
     <row r="212" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A212" s="10" t="s">
@@ -20717,12 +20271,10 @@
         <v>91</v>
       </c>
       <c r="W212" s="10"/>
-      <c r="Z212" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA212" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="Z212" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA212"/>
     </row>
     <row r="213" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A213" s="10" t="s">
@@ -20790,9 +20342,10 @@
         <v>91</v>
       </c>
       <c r="W213" s="10"/>
-      <c r="AA213" s="18" t="s">
-        <v>1647</v>
-      </c>
+      <c r="Z213" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA213"/>
     </row>
     <row r="214" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A214" s="10" t="s">
@@ -20860,9 +20413,7 @@
         <v>149</v>
       </c>
       <c r="W214" s="10"/>
-      <c r="AA214" s="18" t="s">
-        <v>1647</v>
-      </c>
+      <c r="AA214"/>
     </row>
     <row r="215" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A215" s="10" t="s">
@@ -20930,9 +20481,7 @@
         <v>149</v>
       </c>
       <c r="W215" s="10"/>
-      <c r="AA215" s="18" t="s">
-        <v>1647</v>
-      </c>
+      <c r="AA215"/>
     </row>
     <row r="216" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A216" s="10" t="s">
@@ -21000,9 +20549,10 @@
         <v>149</v>
       </c>
       <c r="W216" s="10"/>
-      <c r="AA216" s="18" t="s">
-        <v>1647</v>
-      </c>
+      <c r="Z216" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA216"/>
     </row>
     <row r="217" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A217" s="10" t="s">
@@ -21070,9 +20620,7 @@
         <v>149</v>
       </c>
       <c r="W217" s="10"/>
-      <c r="AA217" s="18" t="s">
-        <v>1647</v>
-      </c>
+      <c r="AA217"/>
     </row>
     <row r="218" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A218" s="10" t="s">
@@ -21140,9 +20688,7 @@
         <v>149</v>
       </c>
       <c r="W218" s="10"/>
-      <c r="AA218" s="18" t="s">
-        <v>1647</v>
-      </c>
+      <c r="AA218"/>
     </row>
     <row r="219" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A219" s="10" t="s">
@@ -21210,9 +20756,7 @@
         <v>149</v>
       </c>
       <c r="W219" s="10"/>
-      <c r="AA219" s="18" t="s">
-        <v>1647</v>
-      </c>
+      <c r="AA219"/>
     </row>
     <row r="220" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A220" s="10" t="s">
@@ -21276,9 +20820,7 @@
         <v>149</v>
       </c>
       <c r="W220" s="10"/>
-      <c r="AA220" s="18" t="s">
-        <v>1647</v>
-      </c>
+      <c r="AA220"/>
     </row>
     <row r="221" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A221" s="10" t="s">
@@ -21346,8 +20888,8 @@
         <v>149</v>
       </c>
       <c r="W221" s="10"/>
-      <c r="AA221" s="18" t="s">
-        <v>1647</v>
+      <c r="AA221" t="s">
+        <v>1643</v>
       </c>
     </row>
     <row r="222" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -21416,9 +20958,7 @@
         <v>149</v>
       </c>
       <c r="W222" s="10"/>
-      <c r="AA222" s="18" t="s">
-        <v>1647</v>
-      </c>
+      <c r="AA222"/>
     </row>
     <row r="223" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A223" s="10" t="s">
@@ -21486,9 +21026,7 @@
         <v>91</v>
       </c>
       <c r="W223" s="10"/>
-      <c r="AA223" s="18" t="s">
-        <v>1647</v>
-      </c>
+      <c r="AA223"/>
     </row>
     <row r="224" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A224" s="10" t="s">
@@ -21556,18 +21094,7 @@
         <v>166</v>
       </c>
       <c r="W224" s="10"/>
-      <c r="X224" s="1" t="s">
-        <v>1641</v>
-      </c>
-      <c r="Y224" s="1" t="s">
-        <v>1641</v>
-      </c>
-      <c r="Z224" s="1" t="s">
-        <v>1641</v>
-      </c>
-      <c r="AA224" s="1" t="s">
-        <v>1641</v>
-      </c>
+      <c r="AA224"/>
     </row>
     <row r="225" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A225" s="10" t="s">
@@ -21635,6 +21162,7 @@
         <v>55</v>
       </c>
       <c r="W225" s="10"/>
+      <c r="AA225"/>
     </row>
     <row r="226" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A226" s="10" t="s">
@@ -21702,6 +21230,7 @@
         <v>166</v>
       </c>
       <c r="W226" s="10"/>
+      <c r="AA226"/>
     </row>
     <row r="227" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A227" s="10" t="s">
@@ -21769,6 +21298,7 @@
         <v>166</v>
       </c>
       <c r="W227" s="10"/>
+      <c r="AA227"/>
     </row>
     <row r="228" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A228" s="10" t="s">
@@ -21836,6 +21366,7 @@
         <v>118</v>
       </c>
       <c r="W228" s="10"/>
+      <c r="AA228"/>
     </row>
     <row r="229" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A229" s="10" t="s">
@@ -21903,6 +21434,9 @@
         <v>118</v>
       </c>
       <c r="W229" s="10"/>
+      <c r="AA229" t="s">
+        <v>1644</v>
+      </c>
     </row>
     <row r="230" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A230" s="10" t="s">
@@ -21970,6 +21504,7 @@
         <v>166</v>
       </c>
       <c r="W230" s="10"/>
+      <c r="AA230"/>
     </row>
     <row r="231" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A231" s="10" t="s">
@@ -22037,6 +21572,7 @@
         <v>149</v>
       </c>
       <c r="W231" s="10"/>
+      <c r="AA231"/>
     </row>
     <row r="232" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A232" s="10" t="s">
@@ -22104,6 +21640,9 @@
         <v>118</v>
       </c>
       <c r="W232" s="10"/>
+      <c r="AA232" t="s">
+        <v>1644</v>
+      </c>
     </row>
     <row r="233" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A233" s="10" t="s">
@@ -22171,12 +21710,7 @@
         <v>118</v>
       </c>
       <c r="W233" s="10"/>
-      <c r="Z233" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA233" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA233"/>
     </row>
     <row r="234" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A234" s="10" t="s">
@@ -22244,12 +21778,7 @@
         <v>118</v>
       </c>
       <c r="W234" s="10"/>
-      <c r="Z234" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA234" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA234"/>
     </row>
     <row r="235" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A235" s="10" t="s">
@@ -22317,12 +21846,7 @@
         <v>118</v>
       </c>
       <c r="W235" s="10"/>
-      <c r="Z235" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA235" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA235"/>
     </row>
     <row r="236" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A236" s="10" t="s">
@@ -22390,6 +21914,9 @@
         <v>118</v>
       </c>
       <c r="W236" s="10"/>
+      <c r="AA236" t="s">
+        <v>1643</v>
+      </c>
     </row>
     <row r="237" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A237" s="10" t="s">
@@ -22457,6 +21984,9 @@
         <v>118</v>
       </c>
       <c r="W237" s="10"/>
+      <c r="AA237" t="s">
+        <v>1643</v>
+      </c>
     </row>
     <row r="238" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A238" s="10" t="s">
@@ -22524,18 +22054,7 @@
         <v>118</v>
       </c>
       <c r="W238" s="10"/>
-      <c r="X238" s="1" t="s">
-        <v>1641</v>
-      </c>
-      <c r="Y238" s="1" t="s">
-        <v>1641</v>
-      </c>
-      <c r="Z238" s="1" t="s">
-        <v>1641</v>
-      </c>
-      <c r="AA238" s="1" t="s">
-        <v>1641</v>
-      </c>
+      <c r="AA238"/>
     </row>
     <row r="239" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A239" s="10" t="s">
@@ -22603,6 +22122,9 @@
         <v>118</v>
       </c>
       <c r="W239" s="10"/>
+      <c r="AA239" t="s">
+        <v>1644</v>
+      </c>
     </row>
     <row r="240" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A240" s="10" t="s">
@@ -22670,6 +22192,9 @@
         <v>118</v>
       </c>
       <c r="W240" s="10"/>
+      <c r="AA240" t="s">
+        <v>1644</v>
+      </c>
     </row>
     <row r="241" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A241" s="10" t="s">
@@ -22737,6 +22262,9 @@
         <v>91</v>
       </c>
       <c r="W241" s="10"/>
+      <c r="AA241" t="s">
+        <v>1644</v>
+      </c>
     </row>
     <row r="242" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A242" s="10" t="s">
@@ -22804,6 +22332,7 @@
         <v>118</v>
       </c>
       <c r="W242" s="10"/>
+      <c r="AA242"/>
     </row>
     <row r="243" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A243" s="10" t="s">
@@ -22871,6 +22400,7 @@
         <v>118</v>
       </c>
       <c r="W243" s="10"/>
+      <c r="AA243"/>
     </row>
     <row r="244" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A244" s="10" t="s">
@@ -22938,6 +22468,7 @@
         <v>149</v>
       </c>
       <c r="W244" s="10"/>
+      <c r="AA244"/>
     </row>
     <row r="245" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A245" s="10" t="s">
@@ -23005,6 +22536,7 @@
         <v>149</v>
       </c>
       <c r="W245" s="10"/>
+      <c r="AA245"/>
     </row>
     <row r="246" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A246" s="10" t="s">
@@ -23072,6 +22604,7 @@
         <v>149</v>
       </c>
       <c r="W246" s="10"/>
+      <c r="AA246"/>
     </row>
     <row r="247" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A247" s="10" t="s">
@@ -23139,6 +22672,10 @@
         <v>149</v>
       </c>
       <c r="W247" s="10"/>
+      <c r="Z247" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA247"/>
     </row>
     <row r="248" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A248" s="10" t="s">
@@ -23206,6 +22743,10 @@
         <v>118</v>
       </c>
       <c r="W248" s="10"/>
+      <c r="Z248" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA248"/>
     </row>
     <row r="249" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A249" s="10" t="s">
@@ -23273,6 +22814,9 @@
         <v>118</v>
       </c>
       <c r="W249" s="10"/>
+      <c r="AA249" t="s">
+        <v>1644</v>
+      </c>
     </row>
     <row r="250" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A250" s="10" t="s">
@@ -23340,6 +22884,7 @@
         <v>118</v>
       </c>
       <c r="W250" s="10"/>
+      <c r="AA250"/>
     </row>
     <row r="251" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A251" s="10" t="s">
@@ -23407,6 +22952,7 @@
         <v>149</v>
       </c>
       <c r="W251" s="10"/>
+      <c r="AA251"/>
     </row>
     <row r="252" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A252" s="10" t="s">
@@ -23474,6 +23020,7 @@
         <v>149</v>
       </c>
       <c r="W252" s="10"/>
+      <c r="AA252"/>
     </row>
     <row r="253" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A253" s="10" t="s">
@@ -23539,6 +23086,10 @@
         <v>149</v>
       </c>
       <c r="W253" s="10"/>
+      <c r="Z253" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA253"/>
     </row>
     <row r="254" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A254" s="10" t="s">
@@ -23606,15 +23157,7 @@
         <v>149</v>
       </c>
       <c r="W254" s="10"/>
-      <c r="X254" s="1" t="s">
-        <v>1643</v>
-      </c>
-      <c r="Y254" s="1" t="s">
-        <v>1644</v>
-      </c>
-      <c r="AA254" s="1" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA254"/>
     </row>
     <row r="255" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A255" s="10" t="s">
@@ -23682,15 +23225,7 @@
         <v>41</v>
       </c>
       <c r="W255" s="10"/>
-      <c r="X255" s="1" t="s">
-        <v>1643</v>
-      </c>
-      <c r="Y255" s="1" t="s">
-        <v>1644</v>
-      </c>
-      <c r="AA255" s="1" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA255"/>
     </row>
     <row r="256" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A256" s="10" t="s">
@@ -23758,12 +23293,7 @@
         <v>149</v>
       </c>
       <c r="W256" s="10"/>
-      <c r="Z256" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA256" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA256"/>
     </row>
     <row r="257" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A257" s="10" t="s">
@@ -23831,12 +23361,7 @@
         <v>149</v>
       </c>
       <c r="W257" s="10"/>
-      <c r="Z257" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA257" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA257"/>
     </row>
     <row r="258" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A258" s="10" t="s">
@@ -23904,6 +23429,7 @@
         <v>149</v>
       </c>
       <c r="W258" s="10"/>
+      <c r="AA258"/>
     </row>
     <row r="259" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A259" s="10" t="s">
@@ -23971,6 +23497,7 @@
         <v>149</v>
       </c>
       <c r="W259" s="10"/>
+      <c r="AA259"/>
     </row>
     <row r="260" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A260" s="10" t="s">
@@ -24038,6 +23565,7 @@
         <v>149</v>
       </c>
       <c r="W260" s="10"/>
+      <c r="AA260"/>
     </row>
     <row r="261" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A261" s="10" t="s">
@@ -24105,6 +23633,10 @@
         <v>149</v>
       </c>
       <c r="W261" s="10"/>
+      <c r="Z261" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA261"/>
     </row>
     <row r="262" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A262" s="10" t="s">
@@ -24172,6 +23704,7 @@
         <v>149</v>
       </c>
       <c r="W262" s="10"/>
+      <c r="AA262"/>
     </row>
     <row r="263" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A263" s="10" t="s">
@@ -24239,6 +23772,7 @@
         <v>149</v>
       </c>
       <c r="W263" s="10"/>
+      <c r="AA263"/>
     </row>
     <row r="264" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A264" s="10" t="s">
@@ -24306,6 +23840,7 @@
         <v>118</v>
       </c>
       <c r="W264" s="10"/>
+      <c r="AA264"/>
     </row>
     <row r="265" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A265" s="10" t="s">
@@ -24373,12 +23908,7 @@
         <v>149</v>
       </c>
       <c r="W265" s="10"/>
-      <c r="Z265" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA265" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA265"/>
     </row>
     <row r="266" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A266" s="10" t="s">
@@ -24446,12 +23976,7 @@
         <v>149</v>
       </c>
       <c r="W266" s="10"/>
-      <c r="Z266" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA266" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA266"/>
     </row>
     <row r="267" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A267" s="10" t="s">
@@ -24519,12 +24044,7 @@
         <v>149</v>
       </c>
       <c r="W267" s="10"/>
-      <c r="Z267" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA267" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA267"/>
     </row>
     <row r="268" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A268" s="10" t="s">
@@ -24592,12 +24112,7 @@
         <v>149</v>
       </c>
       <c r="W268" s="10"/>
-      <c r="Z268" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA268" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA268"/>
     </row>
     <row r="269" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A269" s="10" t="s">
@@ -24665,6 +24180,7 @@
         <v>149</v>
       </c>
       <c r="W269" s="10"/>
+      <c r="AA269"/>
     </row>
     <row r="270" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A270" s="10" t="s">
@@ -24732,6 +24248,9 @@
         <v>55</v>
       </c>
       <c r="W270" s="10"/>
+      <c r="AA270" t="s">
+        <v>1644</v>
+      </c>
     </row>
     <row r="271" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A271" s="10" t="s">
@@ -24799,6 +24318,7 @@
         <v>149</v>
       </c>
       <c r="W271" s="10"/>
+      <c r="AA271"/>
     </row>
     <row r="272" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A272" s="10" t="s">
@@ -24866,6 +24386,7 @@
         <v>149</v>
       </c>
       <c r="W272" s="10"/>
+      <c r="AA272"/>
     </row>
     <row r="273" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A273" s="10" t="s">
@@ -24933,12 +24454,7 @@
         <v>149</v>
       </c>
       <c r="W273" s="10"/>
-      <c r="Z273" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA273" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA273"/>
     </row>
     <row r="274" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A274" s="10" t="s">
@@ -25006,6 +24522,7 @@
         <v>149</v>
       </c>
       <c r="W274" s="10"/>
+      <c r="AA274"/>
     </row>
     <row r="275" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A275" s="10" t="s">
@@ -25073,6 +24590,7 @@
         <v>149</v>
       </c>
       <c r="W275" s="10"/>
+      <c r="AA275"/>
     </row>
     <row r="276" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A276" s="10" t="s">
@@ -25140,6 +24658,7 @@
         <v>149</v>
       </c>
       <c r="W276" s="10"/>
+      <c r="AA276"/>
     </row>
     <row r="277" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A277" s="10" t="s">
@@ -25207,6 +24726,7 @@
         <v>41</v>
       </c>
       <c r="W277" s="10"/>
+      <c r="AA277"/>
     </row>
     <row r="278" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A278" s="10" t="s">
@@ -25274,6 +24794,9 @@
         <v>149</v>
       </c>
       <c r="W278" s="10"/>
+      <c r="AA278" t="s">
+        <v>1644</v>
+      </c>
     </row>
     <row r="279" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A279" s="10" t="s">
@@ -25341,12 +24864,7 @@
         <v>149</v>
       </c>
       <c r="W279" s="10"/>
-      <c r="Z279" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA279" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA279"/>
     </row>
     <row r="280" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A280" s="10" t="s">
@@ -25414,6 +24932,7 @@
         <v>149</v>
       </c>
       <c r="W280" s="10"/>
+      <c r="AA280"/>
     </row>
     <row r="281" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A281" s="10" t="s">
@@ -25481,6 +25000,7 @@
         <v>149</v>
       </c>
       <c r="W281" s="10"/>
+      <c r="AA281"/>
     </row>
     <row r="282" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A282" s="10" t="s">
@@ -25548,6 +25068,7 @@
         <v>149</v>
       </c>
       <c r="W282" s="10"/>
+      <c r="AA282"/>
     </row>
     <row r="283" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A283" s="10" t="s">
@@ -25615,6 +25136,9 @@
         <v>41</v>
       </c>
       <c r="W283" s="10"/>
+      <c r="AA283" t="s">
+        <v>1644</v>
+      </c>
     </row>
     <row r="284" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A284" s="10" t="s">
@@ -25682,6 +25206,7 @@
         <v>149</v>
       </c>
       <c r="W284" s="10"/>
+      <c r="AA284"/>
     </row>
     <row r="285" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A285" s="10" t="s">
@@ -25749,6 +25274,7 @@
         <v>149</v>
       </c>
       <c r="W285" s="10"/>
+      <c r="AA285"/>
     </row>
     <row r="286" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A286" s="10" t="s">
@@ -25816,6 +25342,9 @@
         <v>149</v>
       </c>
       <c r="W286" s="10"/>
+      <c r="AA286" t="s">
+        <v>1644</v>
+      </c>
     </row>
     <row r="287" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A287" s="10" t="s">
@@ -25883,15 +25412,7 @@
         <v>149</v>
       </c>
       <c r="W287" s="10"/>
-      <c r="X287" s="1" t="s">
-        <v>1643</v>
-      </c>
-      <c r="Y287" s="1" t="s">
-        <v>1644</v>
-      </c>
-      <c r="AA287" s="1" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA287"/>
     </row>
     <row r="288" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A288" s="10" t="s">
@@ -25959,12 +25480,7 @@
         <v>149</v>
       </c>
       <c r="W288" s="10"/>
-      <c r="Z288" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA288" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA288"/>
     </row>
     <row r="289" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A289" s="10" t="s">
@@ -26032,6 +25548,7 @@
         <v>41</v>
       </c>
       <c r="W289" s="10"/>
+      <c r="AA289"/>
     </row>
     <row r="290" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A290" s="10" t="s">
@@ -26099,12 +25616,7 @@
         <v>149</v>
       </c>
       <c r="W290" s="10"/>
-      <c r="Z290" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA290" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA290"/>
     </row>
     <row r="291" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A291" s="10" t="s">
@@ -26168,12 +25680,7 @@
         <v>149</v>
       </c>
       <c r="W291" s="10"/>
-      <c r="Z291" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA291" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA291"/>
     </row>
     <row r="292" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A292" s="10" t="s">
@@ -26237,12 +25744,7 @@
         <v>149</v>
       </c>
       <c r="W292" s="10"/>
-      <c r="Z292" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA292" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA292"/>
     </row>
     <row r="293" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A293" s="10" t="s">
@@ -26310,12 +25812,7 @@
         <v>149</v>
       </c>
       <c r="W293" s="10"/>
-      <c r="Z293" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA293" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA293"/>
     </row>
     <row r="294" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A294" s="10" t="s">
@@ -26383,12 +25880,7 @@
         <v>149</v>
       </c>
       <c r="W294" s="10"/>
-      <c r="Z294" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA294" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA294"/>
     </row>
     <row r="295" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A295" s="10" t="s">
@@ -26456,6 +25948,7 @@
         <v>149</v>
       </c>
       <c r="W295" s="10"/>
+      <c r="AA295"/>
     </row>
     <row r="296" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A296" s="10" t="s">
@@ -26523,6 +26016,9 @@
         <v>149</v>
       </c>
       <c r="W296" s="10"/>
+      <c r="AA296" t="s">
+        <v>1644</v>
+      </c>
     </row>
     <row r="297" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A297" s="10" t="s">
@@ -26590,6 +26086,7 @@
         <v>41</v>
       </c>
       <c r="W297" s="10"/>
+      <c r="AA297"/>
     </row>
     <row r="298" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A298" s="10" t="s">
@@ -26657,6 +26154,7 @@
         <v>91</v>
       </c>
       <c r="W298" s="10"/>
+      <c r="AA298"/>
     </row>
     <row r="299" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A299" s="10" t="s">
@@ -26724,6 +26222,7 @@
         <v>149</v>
       </c>
       <c r="W299" s="10"/>
+      <c r="AA299"/>
     </row>
     <row r="300" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A300" s="10" t="s">
@@ -26791,6 +26290,7 @@
         <v>41</v>
       </c>
       <c r="W300" s="10"/>
+      <c r="AA300"/>
     </row>
     <row r="301" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A301" s="10" t="s">
@@ -26858,12 +26358,7 @@
         <v>149</v>
       </c>
       <c r="W301" s="10"/>
-      <c r="Z301" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA301" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA301"/>
     </row>
     <row r="302" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A302" s="10" t="s">
@@ -26931,6 +26426,7 @@
         <v>41</v>
       </c>
       <c r="W302" s="10"/>
+      <c r="AA302"/>
     </row>
     <row r="303" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A303" s="10" t="s">
@@ -26998,6 +26494,7 @@
         <v>91</v>
       </c>
       <c r="W303" s="10"/>
+      <c r="AA303"/>
     </row>
     <row r="304" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A304" s="10" t="s">
@@ -27065,6 +26562,7 @@
         <v>55</v>
       </c>
       <c r="W304" s="10"/>
+      <c r="AA304"/>
     </row>
     <row r="305" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A305" s="10" t="s">
@@ -27128,6 +26626,7 @@
         <v>149</v>
       </c>
       <c r="W305" s="10"/>
+      <c r="AA305"/>
     </row>
     <row r="306" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A306" s="10" t="s">
@@ -27195,6 +26694,7 @@
         <v>91</v>
       </c>
       <c r="W306" s="10"/>
+      <c r="AA306"/>
     </row>
     <row r="307" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A307" s="10" t="s">
@@ -27258,6 +26758,7 @@
         <v>149</v>
       </c>
       <c r="W307" s="10"/>
+      <c r="AA307"/>
     </row>
     <row r="308" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A308" s="10" t="s">
@@ -27321,6 +26822,7 @@
         <v>91</v>
       </c>
       <c r="W308" s="10"/>
+      <c r="AA308"/>
     </row>
     <row r="309" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A309" s="10" t="s">
@@ -27384,6 +26886,7 @@
         <v>41</v>
       </c>
       <c r="W309" s="10"/>
+      <c r="AA309"/>
     </row>
     <row r="310" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A310" s="10" t="s">
@@ -27447,6 +26950,7 @@
         <v>149</v>
       </c>
       <c r="W310" s="10"/>
+      <c r="AA310"/>
     </row>
     <row r="311" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A311" s="10" t="s">
@@ -27514,6 +27018,7 @@
         <v>91</v>
       </c>
       <c r="W311" s="10"/>
+      <c r="AA311"/>
     </row>
     <row r="312" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A312" s="10" t="s">
@@ -27577,6 +27082,7 @@
         <v>149</v>
       </c>
       <c r="W312" s="10"/>
+      <c r="AA312"/>
     </row>
     <row r="313" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A313" s="10" t="s">
@@ -27644,6 +27150,9 @@
         <v>118</v>
       </c>
       <c r="W313" s="10"/>
+      <c r="AA313" t="s">
+        <v>1643</v>
+      </c>
     </row>
     <row r="314" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A314" s="10" t="s">
@@ -27709,9 +27218,7 @@
         <v>166</v>
       </c>
       <c r="W314" s="10"/>
-      <c r="AA314" s="1" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA314"/>
     </row>
     <row r="315" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A315" s="10" t="s">
@@ -27777,9 +27284,7 @@
         <v>166</v>
       </c>
       <c r="W315" s="10"/>
-      <c r="AA315" s="1" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA315"/>
     </row>
     <row r="316" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A316" s="10" t="s">
@@ -27843,9 +27348,7 @@
         <v>149</v>
       </c>
       <c r="W316" s="10"/>
-      <c r="AA316" s="1" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA316"/>
     </row>
     <row r="317" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A317" s="10" t="s">
@@ -27913,6 +27416,7 @@
         <v>149</v>
       </c>
       <c r="W317" s="10"/>
+      <c r="AA317"/>
     </row>
     <row r="318" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A318" s="10" t="s">
@@ -27980,6 +27484,7 @@
         <v>91</v>
       </c>
       <c r="W318" s="10"/>
+      <c r="AA318"/>
     </row>
     <row r="319" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A319" s="10" t="s">
@@ -28047,6 +27552,7 @@
         <v>91</v>
       </c>
       <c r="W319" s="10"/>
+      <c r="AA319"/>
     </row>
     <row r="320" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A320" s="10" t="s">
@@ -28110,12 +27616,7 @@
         <v>41</v>
       </c>
       <c r="W320" s="10"/>
-      <c r="Z320" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA320" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA320"/>
     </row>
     <row r="321" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A321" s="10" t="s">
@@ -28183,6 +27684,9 @@
         <v>91</v>
       </c>
       <c r="W321" s="10"/>
+      <c r="AA321" t="s">
+        <v>1643</v>
+      </c>
     </row>
     <row r="322" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A322" s="10" t="s">
@@ -28246,6 +27750,7 @@
         <v>149</v>
       </c>
       <c r="W322" s="10"/>
+      <c r="AA322"/>
     </row>
     <row r="323" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A323" s="10" t="s">
@@ -28313,6 +27818,7 @@
         <v>91</v>
       </c>
       <c r="W323" s="10"/>
+      <c r="AA323"/>
     </row>
     <row r="324" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A324" s="10" t="s">
@@ -28380,6 +27886,7 @@
         <v>55</v>
       </c>
       <c r="W324" s="10"/>
+      <c r="AA324"/>
     </row>
     <row r="325" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A325" s="10" t="s">
@@ -28443,12 +27950,7 @@
         <v>149</v>
       </c>
       <c r="W325" s="10"/>
-      <c r="Z325" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA325" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA325"/>
     </row>
     <row r="326" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A326" s="10" t="s">
@@ -28516,12 +28018,7 @@
         <v>149</v>
       </c>
       <c r="W326" s="10"/>
-      <c r="Z326" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA326" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA326"/>
     </row>
     <row r="327" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A327" s="10" t="s">
@@ -28585,12 +28082,7 @@
         <v>149</v>
       </c>
       <c r="W327" s="10"/>
-      <c r="Z327" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA327" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA327"/>
     </row>
     <row r="328" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A328" s="10" t="s">
@@ -28658,6 +28150,7 @@
         <v>55</v>
       </c>
       <c r="W328" s="10"/>
+      <c r="AA328"/>
     </row>
     <row r="329" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A329" s="10" t="s">
@@ -28725,6 +28218,7 @@
         <v>55</v>
       </c>
       <c r="W329" s="10"/>
+      <c r="AA329"/>
     </row>
     <row r="330" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A330" s="10" t="s">
@@ -28792,6 +28286,7 @@
         <v>91</v>
       </c>
       <c r="W330" s="10"/>
+      <c r="AA330"/>
     </row>
     <row r="331" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A331" s="10" t="s">
@@ -28859,6 +28354,7 @@
         <v>55</v>
       </c>
       <c r="W331" s="10"/>
+      <c r="AA331"/>
     </row>
     <row r="332" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A332" s="10" t="s">
@@ -28926,6 +28422,7 @@
         <v>41</v>
       </c>
       <c r="W332" s="10"/>
+      <c r="AA332"/>
     </row>
     <row r="333" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A333" s="10" t="s">
@@ -28989,6 +28486,7 @@
         <v>41</v>
       </c>
       <c r="W333" s="10"/>
+      <c r="AA333"/>
     </row>
     <row r="334" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A334" s="10" t="s">
@@ -29056,6 +28554,7 @@
         <v>55</v>
       </c>
       <c r="W334" s="10"/>
+      <c r="AA334"/>
     </row>
     <row r="335" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A335" s="10" t="s">
@@ -29119,6 +28618,7 @@
         <v>91</v>
       </c>
       <c r="W335" s="10"/>
+      <c r="AA335"/>
     </row>
     <row r="336" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A336" s="10" t="s">
@@ -29186,6 +28686,9 @@
         <v>91</v>
       </c>
       <c r="W336" s="10"/>
+      <c r="AA336" t="s">
+        <v>1644</v>
+      </c>
     </row>
     <row r="337" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A337" s="10" t="s">
@@ -29253,6 +28756,7 @@
         <v>91</v>
       </c>
       <c r="W337" s="10"/>
+      <c r="AA337"/>
     </row>
     <row r="338" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A338" s="10" t="s">
@@ -29320,6 +28824,7 @@
         <v>91</v>
       </c>
       <c r="W338" s="10"/>
+      <c r="AA338"/>
     </row>
     <row r="339" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A339" s="10" t="s">
@@ -29387,6 +28892,9 @@
         <v>149</v>
       </c>
       <c r="W339" s="10"/>
+      <c r="AA339" t="s">
+        <v>1643</v>
+      </c>
     </row>
     <row r="340" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A340" s="10" t="s">
@@ -29454,6 +28962,7 @@
         <v>91</v>
       </c>
       <c r="W340" s="10"/>
+      <c r="AA340"/>
     </row>
     <row r="341" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A341" s="10" t="s">
@@ -29521,6 +29030,7 @@
         <v>118</v>
       </c>
       <c r="W341" s="10"/>
+      <c r="AA341"/>
     </row>
     <row r="342" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A342" s="10" t="s">
@@ -29588,6 +29098,7 @@
         <v>91</v>
       </c>
       <c r="W342" s="10"/>
+      <c r="AA342"/>
     </row>
     <row r="343" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A343" s="10" t="s">
@@ -29655,6 +29166,10 @@
         <v>91</v>
       </c>
       <c r="W343" s="10"/>
+      <c r="Z343" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA343"/>
     </row>
     <row r="344" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A344" s="10" t="s">
@@ -29722,6 +29237,10 @@
         <v>91</v>
       </c>
       <c r="W344" s="10"/>
+      <c r="Z344" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA344"/>
     </row>
     <row r="345" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A345" s="10" t="s">
@@ -29785,6 +29304,7 @@
         <v>55</v>
       </c>
       <c r="W345" s="10"/>
+      <c r="AA345"/>
     </row>
     <row r="346" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A346" s="10" t="s">
@@ -29848,6 +29368,10 @@
         <v>118</v>
       </c>
       <c r="W346" s="10"/>
+      <c r="Z346" t="s">
+        <v>1643</v>
+      </c>
+      <c r="AA346"/>
     </row>
     <row r="347" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A347" s="10" t="s">
@@ -29915,6 +29439,7 @@
         <v>149</v>
       </c>
       <c r="W347" s="10"/>
+      <c r="AA347"/>
     </row>
     <row r="348" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A348" s="10" t="s">
@@ -29982,6 +29507,7 @@
         <v>149</v>
       </c>
       <c r="W348" s="10"/>
+      <c r="AA348"/>
     </row>
     <row r="349" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A349" s="10" t="s">
@@ -30045,17 +29571,10 @@
         <v>166</v>
       </c>
       <c r="W349" s="10"/>
-      <c r="X349" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="Y349" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="Z349" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA349" s="18" t="s">
-        <v>1642</v>
+      <c r="X349" s="18"/>
+      <c r="Y349" s="18"/>
+      <c r="AA349" t="s">
+        <v>1644</v>
       </c>
     </row>
     <row r="350" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -30124,18 +29643,7 @@
         <v>149</v>
       </c>
       <c r="W350" s="10"/>
-      <c r="X350" s="1" t="s">
-        <v>1641</v>
-      </c>
-      <c r="Y350" s="1" t="s">
-        <v>1641</v>
-      </c>
-      <c r="Z350" s="1" t="s">
-        <v>1641</v>
-      </c>
-      <c r="AA350" s="1" t="s">
-        <v>1641</v>
-      </c>
+      <c r="AA350"/>
     </row>
     <row r="351" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A351" s="10" t="s">
@@ -30203,18 +29711,7 @@
         <v>91</v>
       </c>
       <c r="W351" s="10"/>
-      <c r="X351" s="1" t="s">
-        <v>1641</v>
-      </c>
-      <c r="Y351" s="1" t="s">
-        <v>1641</v>
-      </c>
-      <c r="Z351" s="1" t="s">
-        <v>1641</v>
-      </c>
-      <c r="AA351" s="1" t="s">
-        <v>1641</v>
-      </c>
+      <c r="AA351"/>
     </row>
     <row r="352" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A352" s="10" t="s">
@@ -30278,6 +29775,7 @@
         <v>149</v>
       </c>
       <c r="W352" s="10"/>
+      <c r="AA352"/>
     </row>
     <row r="353" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A353" s="10" t="s">
@@ -30341,6 +29839,7 @@
         <v>149</v>
       </c>
       <c r="W353" s="10"/>
+      <c r="AA353"/>
     </row>
     <row r="354" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A354" s="10" t="s">
@@ -30408,6 +29907,7 @@
         <v>149</v>
       </c>
       <c r="W354" s="10"/>
+      <c r="AA354"/>
     </row>
     <row r="355" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A355" s="10" t="s">
@@ -30475,6 +29975,9 @@
         <v>91</v>
       </c>
       <c r="W355" s="10"/>
+      <c r="AA355" t="s">
+        <v>1644</v>
+      </c>
     </row>
     <row r="356" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A356" s="10" t="s">
@@ -30538,12 +30041,7 @@
         <v>149</v>
       </c>
       <c r="W356" s="10"/>
-      <c r="Z356" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA356" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA356"/>
     </row>
     <row r="357" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A357" s="10" t="s">
@@ -30607,6 +30105,7 @@
         <v>149</v>
       </c>
       <c r="W357" s="10"/>
+      <c r="AA357"/>
     </row>
     <row r="358" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A358" s="10" t="s">
@@ -30674,6 +30173,9 @@
         <v>55</v>
       </c>
       <c r="W358" s="10"/>
+      <c r="AA358" t="s">
+        <v>1643</v>
+      </c>
     </row>
     <row r="359" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A359" s="10" t="s">
@@ -30737,6 +30239,9 @@
         <v>55</v>
       </c>
       <c r="W359" s="10"/>
+      <c r="AA359" t="s">
+        <v>1643</v>
+      </c>
     </row>
     <row r="360" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A360" s="10" t="s">
@@ -30804,6 +30309,9 @@
         <v>91</v>
       </c>
       <c r="W360" s="10"/>
+      <c r="AA360" t="s">
+        <v>1643</v>
+      </c>
     </row>
     <row r="361" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A361" s="10" t="s">
@@ -30871,6 +30379,9 @@
         <v>55</v>
       </c>
       <c r="W361" s="10"/>
+      <c r="AA361" t="s">
+        <v>1643</v>
+      </c>
     </row>
     <row r="362" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A362" s="10" t="s">
@@ -30938,6 +30449,9 @@
         <v>55</v>
       </c>
       <c r="W362" s="10"/>
+      <c r="AA362" t="s">
+        <v>1643</v>
+      </c>
     </row>
     <row r="363" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A363" s="10" t="s">
@@ -31005,6 +30519,9 @@
         <v>55</v>
       </c>
       <c r="W363" s="10"/>
+      <c r="AA363" t="s">
+        <v>1643</v>
+      </c>
     </row>
     <row r="364" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A364" s="10" t="s">
@@ -31072,6 +30589,9 @@
         <v>55</v>
       </c>
       <c r="W364" s="10"/>
+      <c r="AA364" t="s">
+        <v>1643</v>
+      </c>
     </row>
     <row r="365" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A365" s="10" t="s">
@@ -31137,6 +30657,9 @@
         <v>149</v>
       </c>
       <c r="W365" s="10"/>
+      <c r="AA365" t="s">
+        <v>1644</v>
+      </c>
     </row>
     <row r="366" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A366" s="10" t="s">
@@ -31200,6 +30723,7 @@
         <v>91</v>
       </c>
       <c r="W366" s="10"/>
+      <c r="AA366"/>
     </row>
     <row r="367" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A367" s="10" t="s">
@@ -31267,6 +30791,7 @@
         <v>41</v>
       </c>
       <c r="W367" s="10"/>
+      <c r="AA367"/>
     </row>
     <row r="368" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A368" s="10" t="s">
@@ -31334,6 +30859,7 @@
         <v>149</v>
       </c>
       <c r="W368" s="10"/>
+      <c r="AA368"/>
     </row>
     <row r="369" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A369" s="10" t="s">
@@ -31401,6 +30927,7 @@
         <v>91</v>
       </c>
       <c r="W369" s="10"/>
+      <c r="AA369"/>
     </row>
     <row r="370" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A370" s="10" t="s">
@@ -31468,6 +30995,7 @@
         <v>149</v>
       </c>
       <c r="W370" s="10"/>
+      <c r="AA370"/>
     </row>
     <row r="371" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A371" s="10" t="s">
@@ -31535,6 +31063,7 @@
         <v>91</v>
       </c>
       <c r="W371" s="10"/>
+      <c r="AA371"/>
     </row>
     <row r="372" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A372" s="10" t="s">
@@ -31598,6 +31127,7 @@
         <v>149</v>
       </c>
       <c r="W372" s="10"/>
+      <c r="AA372"/>
     </row>
     <row r="373" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A373" s="10" t="s">
@@ -31665,6 +31195,7 @@
         <v>149</v>
       </c>
       <c r="W373" s="10"/>
+      <c r="AA373"/>
     </row>
     <row r="374" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A374" s="10" t="s">
@@ -31732,6 +31263,7 @@
         <v>91</v>
       </c>
       <c r="W374" s="10"/>
+      <c r="AA374"/>
     </row>
     <row r="375" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A375" s="10" t="s">
@@ -31795,6 +31327,7 @@
         <v>149</v>
       </c>
       <c r="W375" s="10"/>
+      <c r="AA375"/>
     </row>
     <row r="376" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A376" s="10" t="s">
@@ -31862,6 +31395,9 @@
         <v>55</v>
       </c>
       <c r="W376" s="10"/>
+      <c r="AA376" t="s">
+        <v>1644</v>
+      </c>
     </row>
     <row r="377" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A377" s="10" t="s">
@@ -31929,6 +31465,9 @@
         <v>55</v>
       </c>
       <c r="W377" s="10"/>
+      <c r="AA377" t="s">
+        <v>1643</v>
+      </c>
     </row>
     <row r="378" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A378" s="10" t="s">
@@ -31996,12 +31535,7 @@
         <v>149</v>
       </c>
       <c r="W378" s="10"/>
-      <c r="Z378" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA378" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA378"/>
     </row>
     <row r="379" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A379" s="10" t="s">
@@ -32069,6 +31603,7 @@
         <v>91</v>
       </c>
       <c r="W379" s="10"/>
+      <c r="AA379"/>
     </row>
     <row r="380" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A380" s="10" t="s">
@@ -32132,6 +31667,9 @@
         <v>149</v>
       </c>
       <c r="W380" s="10"/>
+      <c r="AA380" t="s">
+        <v>1644</v>
+      </c>
     </row>
     <row r="381" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A381" s="10" t="s">
@@ -32199,6 +31737,7 @@
         <v>91</v>
       </c>
       <c r="W381" s="10"/>
+      <c r="AA381"/>
     </row>
     <row r="382" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A382" s="10" t="s">
@@ -32266,6 +31805,7 @@
         <v>91</v>
       </c>
       <c r="W382" s="10"/>
+      <c r="AA382"/>
     </row>
     <row r="383" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A383" s="10" t="s">
@@ -32329,6 +31869,7 @@
         <v>91</v>
       </c>
       <c r="W383" s="10"/>
+      <c r="AA383"/>
     </row>
     <row r="384" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A384" s="10" t="s">
@@ -32392,8 +31933,9 @@
         <v>91</v>
       </c>
       <c r="W384" s="10"/>
-    </row>
-    <row r="385" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AA384"/>
+    </row>
+    <row r="385" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A385" s="10" t="s">
         <v>1518</v>
       </c>
@@ -32459,8 +32001,11 @@
         <v>166</v>
       </c>
       <c r="W385" s="10"/>
-    </row>
-    <row r="386" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AA385" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="386" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A386" s="10" t="s">
         <v>1523</v>
       </c>
@@ -32522,8 +32067,9 @@
         <v>91</v>
       </c>
       <c r="W386" s="10"/>
-    </row>
-    <row r="387" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AA386"/>
+    </row>
+    <row r="387" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A387" s="10" t="s">
         <v>1525</v>
       </c>
@@ -32585,8 +32131,9 @@
         <v>91</v>
       </c>
       <c r="W387" s="10"/>
-    </row>
-    <row r="388" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AA387"/>
+    </row>
+    <row r="388" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A388" s="10" t="s">
         <v>1527</v>
       </c>
@@ -32648,8 +32195,9 @@
         <v>91</v>
       </c>
       <c r="W388" s="10"/>
-    </row>
-    <row r="389" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AA388"/>
+    </row>
+    <row r="389" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A389" s="10" t="s">
         <v>1529</v>
       </c>
@@ -32711,8 +32259,9 @@
         <v>91</v>
       </c>
       <c r="W389" s="10"/>
-    </row>
-    <row r="390" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AA389"/>
+    </row>
+    <row r="390" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A390" s="10" t="s">
         <v>1531</v>
       </c>
@@ -32776,8 +32325,9 @@
         <v>91</v>
       </c>
       <c r="W390" s="10"/>
-    </row>
-    <row r="391" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AA390"/>
+    </row>
+    <row r="391" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A391" s="10" t="s">
         <v>989</v>
       </c>
@@ -32843,8 +32393,9 @@
         <v>149</v>
       </c>
       <c r="W391" s="10"/>
-    </row>
-    <row r="392" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AA391"/>
+    </row>
+    <row r="392" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A392" s="10" t="s">
         <v>1537</v>
       </c>
@@ -32910,8 +32461,9 @@
         <v>91</v>
       </c>
       <c r="W392" s="10"/>
-    </row>
-    <row r="393" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AA392"/>
+    </row>
+    <row r="393" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A393" s="10" t="s">
         <v>1540</v>
       </c>
@@ -32977,8 +32529,11 @@
         <v>166</v>
       </c>
       <c r="W393" s="10"/>
-    </row>
-    <row r="394" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AA393" t="s">
+        <v>1643</v>
+      </c>
+    </row>
+    <row r="394" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A394" s="10" t="s">
         <v>1546</v>
       </c>
@@ -33044,8 +32599,9 @@
         <v>91</v>
       </c>
       <c r="W394" s="10"/>
-    </row>
-    <row r="395" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AA394"/>
+    </row>
+    <row r="395" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A395" s="10" t="s">
         <v>1550</v>
       </c>
@@ -33111,8 +32667,9 @@
         <v>149</v>
       </c>
       <c r="W395" s="10"/>
-    </row>
-    <row r="396" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AA395"/>
+    </row>
+    <row r="396" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A396" s="10" t="s">
         <v>1553</v>
       </c>
@@ -33178,8 +32735,9 @@
         <v>149</v>
       </c>
       <c r="W396" s="10"/>
-    </row>
-    <row r="397" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AA396"/>
+    </row>
+    <row r="397" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A397" s="10" t="s">
         <v>1559</v>
       </c>
@@ -33245,8 +32803,9 @@
         <v>166</v>
       </c>
       <c r="W397" s="10"/>
-    </row>
-    <row r="398" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AA397"/>
+    </row>
+    <row r="398" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A398" s="10" t="s">
         <v>1562</v>
       </c>
@@ -33312,8 +32871,9 @@
         <v>91</v>
       </c>
       <c r="W398" s="10"/>
-    </row>
-    <row r="399" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AA398"/>
+    </row>
+    <row r="399" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A399" s="10" t="s">
         <v>1568</v>
       </c>
@@ -33375,8 +32935,9 @@
         <v>91</v>
       </c>
       <c r="W399" s="10"/>
-    </row>
-    <row r="400" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AA399"/>
+    </row>
+    <row r="400" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A400" s="10" t="s">
         <v>1570</v>
       </c>
@@ -33442,6 +33003,7 @@
         <v>91</v>
       </c>
       <c r="W400" s="10"/>
+      <c r="AA400"/>
     </row>
     <row r="401" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A401" s="10" t="s">
@@ -33505,6 +33067,7 @@
         <v>55</v>
       </c>
       <c r="W401" s="10"/>
+      <c r="AA401"/>
     </row>
     <row r="402" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A402" s="10" t="s">
@@ -33568,6 +33131,7 @@
         <v>166</v>
       </c>
       <c r="W402" s="10"/>
+      <c r="AA402"/>
     </row>
     <row r="403" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A403" s="10" t="s">
@@ -33631,6 +33195,7 @@
         <v>149</v>
       </c>
       <c r="W403" s="10"/>
+      <c r="AA403"/>
     </row>
     <row r="404" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A404" s="10" t="s">
@@ -33698,6 +33263,7 @@
         <v>149</v>
       </c>
       <c r="W404" s="10"/>
+      <c r="AA404"/>
     </row>
     <row r="405" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A405" s="10" t="s">
@@ -33761,6 +33327,7 @@
         <v>149</v>
       </c>
       <c r="W405" s="10"/>
+      <c r="AA405"/>
     </row>
     <row r="406" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A406" s="10" t="s">
@@ -33828,6 +33395,7 @@
         <v>149</v>
       </c>
       <c r="W406" s="10"/>
+      <c r="AA406"/>
     </row>
     <row r="407" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A407" s="10" t="s">
@@ -33895,6 +33463,7 @@
         <v>166</v>
       </c>
       <c r="W407" s="10"/>
+      <c r="AA407"/>
     </row>
     <row r="408" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A408" s="10" t="s">
@@ -33962,18 +33531,7 @@
         <v>91</v>
       </c>
       <c r="W408" s="10"/>
-      <c r="X408" s="1" t="s">
-        <v>1641</v>
-      </c>
-      <c r="Y408" s="1" t="s">
-        <v>1641</v>
-      </c>
-      <c r="Z408" s="1" t="s">
-        <v>1641</v>
-      </c>
-      <c r="AA408" s="1" t="s">
-        <v>1641</v>
-      </c>
+      <c r="AA408"/>
     </row>
     <row r="409" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A409" s="10" t="s">
@@ -34041,6 +33599,9 @@
         <v>118</v>
       </c>
       <c r="W409" s="10"/>
+      <c r="AA409" t="s">
+        <v>1644</v>
+      </c>
     </row>
     <row r="410" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A410" s="10" t="s">
@@ -34108,12 +33669,7 @@
         <v>118</v>
       </c>
       <c r="W410" s="10"/>
-      <c r="Z410" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA410" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA410"/>
     </row>
     <row r="411" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A411" s="10" t="s">
@@ -34177,12 +33733,7 @@
         <v>91</v>
       </c>
       <c r="W411" s="10"/>
-      <c r="Z411" s="18" t="s">
-        <v>1647</v>
-      </c>
-      <c r="AA411" s="18" t="s">
-        <v>1642</v>
-      </c>
+      <c r="AA411"/>
     </row>
     <row r="412" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A412" s="10" t="s">
@@ -34250,6 +33801,9 @@
         <v>91</v>
       </c>
       <c r="W412" s="10"/>
+      <c r="AA412" t="s">
+        <v>1644</v>
+      </c>
     </row>
     <row r="413" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A413" s="10" t="s">
@@ -34317,6 +33871,7 @@
         <v>149</v>
       </c>
       <c r="W413" s="10"/>
+      <c r="AA413"/>
     </row>
     <row r="414" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A414" s="10" t="s">
@@ -34384,6 +33939,7 @@
         <v>149</v>
       </c>
       <c r="W414" s="10"/>
+      <c r="AA414"/>
     </row>
     <row r="415" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A415" s="15" t="s">
@@ -34451,6 +34007,9 @@
         <v>91</v>
       </c>
       <c r="W415" s="15"/>
+      <c r="AA415" t="s">
+        <v>1643</v>
+      </c>
     </row>
     <row r="416" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A416" s="5" t="s">
@@ -34519,7 +34078,7 @@
       </c>
       <c r="W416" s="5"/>
     </row>
-    <row r="417" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="417" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A417" s="5" t="s">
         <v>1631</v>
       </c>
@@ -34583,8 +34142,9 @@
         <v>149</v>
       </c>
       <c r="W417" s="5"/>
-    </row>
-    <row r="418" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AA417" s="18"/>
+    </row>
+    <row r="418" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A418" s="5" t="s">
         <v>1634</v>
       </c>
@@ -34651,7 +34211,7 @@
       </c>
       <c r="W418" s="5"/>
     </row>
-    <row r="419" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="419" spans="1:27" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A419"/>
     </row>
   </sheetData>
@@ -34685,80 +34245,21 @@
   </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="O8" r:id="rId1" xr:uid="{FE12D687-3A50-4D67-B86E-18B9C91A618D}"/>
-    <hyperlink ref="AA2" r:id="rId2" xr:uid="{40BD019B-4ED6-4039-850C-071EADC01DBB}"/>
-    <hyperlink ref="X3" r:id="rId3" xr:uid="{ECDB2A23-869A-4AB3-AE5F-902A20F73367}"/>
-    <hyperlink ref="Y3" r:id="rId4" xr:uid="{F8F61405-927B-4626-A71E-3F08AB8E26E9}"/>
-    <hyperlink ref="Z3" r:id="rId5" xr:uid="{5E188B67-3273-44D2-B02F-39875B64C496}"/>
-    <hyperlink ref="X349" r:id="rId6" xr:uid="{1D25AA0D-9ED5-462C-9B17-78E0E0CFCB05}"/>
-    <hyperlink ref="Y349:Z349" r:id="rId7" display="nicolas.cavalcante@flytour.com.br" xr:uid="{0BCD8A21-DD0F-4C4C-95A2-4CE9FE7B827B}"/>
-    <hyperlink ref="AA349" r:id="rId8" xr:uid="{451A5A85-78EA-44A0-8985-B7044E5F87F6}"/>
-    <hyperlink ref="Z2" r:id="rId9" xr:uid="{EA5D7863-97AA-4A79-B2FA-42E9719440EC}"/>
-    <hyperlink ref="Z18:Z19" r:id="rId10" display="nicolas.cavalcante@flytour.com.br" xr:uid="{4FBED6A0-AE1F-4567-8337-1378351FAD0B}"/>
-    <hyperlink ref="Z41" r:id="rId11" xr:uid="{55763C91-4A00-4D5E-AEF9-BEF4007E634C}"/>
-    <hyperlink ref="Z50" r:id="rId12" xr:uid="{331AA761-EB4B-4314-980C-7F79A03D35A9}"/>
-    <hyperlink ref="Z69" r:id="rId13" xr:uid="{0DFD3848-E447-490E-8411-4F2453ECFA6A}"/>
-    <hyperlink ref="Z175" r:id="rId14" xr:uid="{EE4C1CED-7A9E-4A04-83A6-CAA230AEB07F}"/>
-    <hyperlink ref="Z178" r:id="rId15" xr:uid="{5F329722-922F-43A3-A095-EF7882BCCFD4}"/>
-    <hyperlink ref="Z180" r:id="rId16" xr:uid="{3290402F-A5D7-4CBA-B102-2F9FFDA3B1E0}"/>
-    <hyperlink ref="Z194:Z196" r:id="rId17" display="nicolas.cavalcante@flytour.com.br" xr:uid="{F44C73FF-F1C5-4899-84AA-DD5EC9D40965}"/>
-    <hyperlink ref="Z203" r:id="rId18" xr:uid="{5F964F99-3372-4282-8238-D2F14763958D}"/>
-    <hyperlink ref="Z206" r:id="rId19" xr:uid="{3D9F5FFC-F112-4B18-AE2C-E7A8C04F6F5E}"/>
-    <hyperlink ref="Z212" r:id="rId20" xr:uid="{4D91306B-F86C-4807-97F0-37B515972E33}"/>
-    <hyperlink ref="Z233:Z235" r:id="rId21" display="nicolas.cavalcante@flytour.com.br" xr:uid="{2FC92E5A-37B8-44E9-9665-AD4A08E3F7FF}"/>
-    <hyperlink ref="Z256:Z257" r:id="rId22" display="nicolas.cavalcante@flytour.com.br" xr:uid="{39B596CE-15F8-484B-9B74-F22F40916A3B}"/>
-    <hyperlink ref="Z265:Z268" r:id="rId23" display="nicolas.cavalcante@flytour.com.br" xr:uid="{94F0B865-F78A-4D8D-B645-01F990885EB7}"/>
-    <hyperlink ref="Z273" r:id="rId24" xr:uid="{C909DC1D-4FC5-4626-B381-39783C5889B3}"/>
-    <hyperlink ref="Z279" r:id="rId25" xr:uid="{1DCFF01E-F96A-42E7-9FDA-C09457200AC9}"/>
-    <hyperlink ref="Z288" r:id="rId26" xr:uid="{CE638E84-F129-4074-8DED-B84EB8DD4826}"/>
-    <hyperlink ref="Z290:Z294" r:id="rId27" display="nicolas.cavalcante@flytour.com.br" xr:uid="{86BA15F8-107E-4974-BACE-C7DF3C479B7F}"/>
-    <hyperlink ref="Z301" r:id="rId28" xr:uid="{9A478497-46B6-4020-B00C-534155D0AE25}"/>
-    <hyperlink ref="Z320" r:id="rId29" xr:uid="{AF55BF44-7820-4219-8B5C-9A19548AD495}"/>
-    <hyperlink ref="Z325:Z327" r:id="rId30" display="nicolas.cavalcante@flytour.com.br" xr:uid="{6730F6F7-71AD-4F6D-A3E0-322569163303}"/>
-    <hyperlink ref="Z356" r:id="rId31" xr:uid="{F159F5A6-6E8F-488B-96E1-AD7232BCDA4C}"/>
-    <hyperlink ref="Z378" r:id="rId32" xr:uid="{6463BB10-495E-47AA-AF2D-D40658C5497A}"/>
-    <hyperlink ref="Z410:Z411" r:id="rId33" display="nicolas.cavalcante@flytour.com.br" xr:uid="{0437B841-F89F-4C38-BD51-70F496F5ABBB}"/>
-    <hyperlink ref="Z4" r:id="rId34" xr:uid="{3DD8D310-580C-4DCA-B42D-976AD5C4DD20}"/>
-    <hyperlink ref="Z5" r:id="rId35" xr:uid="{56252C5D-4FE9-48F3-AC24-98C9108BC633}"/>
-    <hyperlink ref="Z6" r:id="rId36" xr:uid="{BCC6CEBD-DDF0-4DA7-9455-DDF0C42D82B0}"/>
-    <hyperlink ref="Z7" r:id="rId37" xr:uid="{5E1A7A27-A2D8-4606-8D2B-9C6DAA0C21F0}"/>
-    <hyperlink ref="Z8" r:id="rId38" xr:uid="{12665683-956D-45AF-BED7-D2A77C975DB2}"/>
-    <hyperlink ref="Z9" r:id="rId39" xr:uid="{DE46BC45-D516-4168-B563-5532906D63D5}"/>
-    <hyperlink ref="Z10" r:id="rId40" xr:uid="{01C5E2D4-A00C-473B-B438-031ABF229367}"/>
-    <hyperlink ref="Z11" r:id="rId41" xr:uid="{7A1A85F5-D7B6-4F12-A833-DCAA77A8C840}"/>
-    <hyperlink ref="Z12" r:id="rId42" xr:uid="{FFC1A7AD-1087-41D3-8893-C62916767588}"/>
-    <hyperlink ref="Z13" r:id="rId43" xr:uid="{08630CE9-5BE4-4F91-B45D-C578D58A70C1}"/>
-    <hyperlink ref="Z14" r:id="rId44" xr:uid="{EB073232-D60A-47E0-8087-DE0C7A7104ED}"/>
-    <hyperlink ref="Z15" r:id="rId45" xr:uid="{68A11C68-6B04-418C-9329-7B6324E41A7B}"/>
-    <hyperlink ref="Z16" r:id="rId46" xr:uid="{75568C17-6FED-4395-8FFA-F1E5914D9FFF}"/>
-    <hyperlink ref="Z17" r:id="rId47" xr:uid="{75152D93-A994-407C-B484-748456DCAD18}"/>
-    <hyperlink ref="AA20" r:id="rId48" xr:uid="{61F487E3-3A31-4330-BD31-98E3C43F7EB8}"/>
-    <hyperlink ref="AA21:AA40" r:id="rId49" display="nicolas.cavalcante@flytour.com.br" xr:uid="{B5112300-9AE1-456A-9E6D-FF116809D583}"/>
-    <hyperlink ref="AA42:AA49" r:id="rId50" display="nicolas.cavalcante@flytour.com.br" xr:uid="{CB74D664-7DB0-434E-994A-A1DC8806E488}"/>
-    <hyperlink ref="AA51:AA68" r:id="rId51" display="nicolas.cavalcante@flytour.com.br" xr:uid="{A320ACC5-BDE8-406E-B25B-10C0CC6517C8}"/>
-    <hyperlink ref="AA197" r:id="rId52" xr:uid="{D30E118D-45C2-4553-9370-508A7337A049}"/>
-    <hyperlink ref="AA198:AA203" r:id="rId53" display="nicolas.cavalcante@flytour.com.br" xr:uid="{D6F39C22-F158-4A52-A1F7-C455D4A195D3}"/>
-    <hyperlink ref="AA204:AA205" r:id="rId54" display="nicolas.cavalcante@flytour.com.br" xr:uid="{44B1C87C-5D5D-4C72-A9FB-BB62ACC17440}"/>
-    <hyperlink ref="AA207:AA211" r:id="rId55" display="nicolas.cavalcante@flytour.com.br" xr:uid="{6F77ED04-00B2-4DB4-BA5B-7A280D6DB164}"/>
-    <hyperlink ref="AA213:AA223" r:id="rId56" display="nicolas.cavalcante@flytour.com.br" xr:uid="{3128AEED-D236-40A9-9207-5C6A648965D9}"/>
-    <hyperlink ref="AA4:AA19" r:id="rId57" display="allan.ribeiro@flytour.com.br" xr:uid="{2FA34CC0-27F0-4713-84CD-4B39C511DCC5}"/>
-    <hyperlink ref="AA41" r:id="rId58" xr:uid="{B0C92966-DEE4-4D36-8005-82ACEF506907}"/>
-    <hyperlink ref="AA50" r:id="rId59" xr:uid="{4277A3FF-AB2C-4C5C-818D-C7E5C020570E}"/>
-    <hyperlink ref="AA69:AA196" r:id="rId60" display="allan.ribeiro@flytour.com.br" xr:uid="{F700B0DC-8A5E-4E7A-A740-927EBA7E13AD}"/>
-    <hyperlink ref="AA206" r:id="rId61" xr:uid="{40D2324D-0501-4D9D-8A4A-E8BAED80D0EA}"/>
-    <hyperlink ref="AA212" r:id="rId62" xr:uid="{FCFD4F02-250A-4C36-B274-8D15B5C6A9FE}"/>
-    <hyperlink ref="AA233:AA235" r:id="rId63" display="allan.ribeiro@flytour.com.br" xr:uid="{62865395-72E2-4BA5-813E-07C58AC07D04}"/>
-    <hyperlink ref="AA256:AA257" r:id="rId64" display="allan.ribeiro@flytour.com.br" xr:uid="{5F4260D5-13DA-42E9-95CA-FD13E34B1BC9}"/>
-    <hyperlink ref="AA265:AA268" r:id="rId65" display="allan.ribeiro@flytour.com.br" xr:uid="{AA463B16-BDDF-4119-8907-867BD0904F8C}"/>
-    <hyperlink ref="AA273" r:id="rId66" xr:uid="{9368C10D-5678-4726-98C0-BCDA9752F23D}"/>
-    <hyperlink ref="AA279" r:id="rId67" xr:uid="{0777998F-FC64-4964-9949-7864D9F23341}"/>
-    <hyperlink ref="AA288" r:id="rId68" xr:uid="{E5996728-E055-4A41-B358-84EF2FE7B79C}"/>
-    <hyperlink ref="AA290:AA294" r:id="rId69" display="allan.ribeiro@flytour.com.br" xr:uid="{AA694B50-AFED-4E6A-924E-FE2EDCC4ADCD}"/>
-    <hyperlink ref="AA301" r:id="rId70" xr:uid="{2F9CC6B3-DE5D-47E9-ABF5-876B406EC5CC}"/>
-    <hyperlink ref="AA320" r:id="rId71" xr:uid="{173D0130-6C6B-4FCD-B83A-6359E27AC916}"/>
-    <hyperlink ref="AA325:AA327" r:id="rId72" display="allan.ribeiro@flytour.com.br" xr:uid="{883B2F67-B511-49F7-8D43-DC82CB86E3DB}"/>
-    <hyperlink ref="AA356" r:id="rId73" xr:uid="{D7A83F70-4159-4E63-ADC7-70D1334C9468}"/>
-    <hyperlink ref="AA378" r:id="rId74" xr:uid="{53EB3276-5FFF-42AE-840F-A89E783BD9BA}"/>
-    <hyperlink ref="AA410:AA411" r:id="rId75" display="allan.ribeiro@flytour.com.br" xr:uid="{E314DF4B-8750-4839-8FA3-2C9438B70671}"/>
+    <hyperlink ref="Y349:Z349" r:id="rId2" display="nicolas.cavalcante@flytour.com.br" xr:uid="{0BCD8A21-DD0F-4C4C-95A2-4CE9FE7B827B}"/>
+    <hyperlink ref="AA80" r:id="rId3" xr:uid="{8058EDCC-447F-4F69-84EC-343CF55ABEA1}"/>
+    <hyperlink ref="AA103:AA104" r:id="rId4" display="nicolas.cavalcante@flytour.com.br" xr:uid="{7489CB4B-3D3B-43CC-B738-20DB2460DD61}"/>
+    <hyperlink ref="AA109:AA110" r:id="rId5" display="nicolas.cavalcante@flytour.com.br" xr:uid="{88EC3E66-CBBA-4188-AD09-18E4E1BEF457}"/>
+    <hyperlink ref="AA134" r:id="rId6" xr:uid="{193F7217-35D8-4BAE-9D80-3617F270A90A}"/>
+    <hyperlink ref="AA185" r:id="rId7" xr:uid="{95A8AFFF-A35A-4EC9-BECD-5B49F22EC8CB}"/>
+    <hyperlink ref="AA221" r:id="rId8" xr:uid="{938752C0-638E-4C4B-900E-9CF1E96CA090}"/>
+    <hyperlink ref="AA236:AA237" r:id="rId9" display="nicolas.cavalcante@flytour.com.br" xr:uid="{072AFFE6-174E-453E-B233-F07EDCF01AD3}"/>
+    <hyperlink ref="AA313" r:id="rId10" xr:uid="{31106F16-6B3D-4DB6-87A9-764E009E5EFF}"/>
+    <hyperlink ref="AA321" r:id="rId11" xr:uid="{45732C80-27F5-4A2B-BD6F-F72F239B56A6}"/>
+    <hyperlink ref="AA339" r:id="rId12" xr:uid="{082FA64A-8359-46E2-92E4-810B6301493E}"/>
+    <hyperlink ref="AA358:AA364" r:id="rId13" display="nicolas.cavalcante@flytour.com.br" xr:uid="{D8D43A6A-560F-497B-8966-AD303710B7F5}"/>
+    <hyperlink ref="AA377" r:id="rId14" xr:uid="{3DBB5404-2833-4749-947E-4FB13E75EA85}"/>
+    <hyperlink ref="AA393" r:id="rId15" xr:uid="{D893AD68-CFE0-4968-8626-A4282F57C801}"/>
+    <hyperlink ref="AA415" r:id="rId16" xr:uid="{162A3F60-6B08-4DD1-AB10-479AFCABB0BF}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>